<commit_message>
Update reports and add new PDF and Excel files
Updated several existing Excel reports and added new reports for ZUPPER VIAGENS and multiple PDF files for September and October 2025. These changes expand the available data and keep existing reports up to date.
</commit_message>
<xml_diff>
--- a/Integration-Quality/EMPRESAS/Relatorio - KONTRIP VIAGENS.xlsx
+++ b/Integration-Quality/EMPRESAS/Relatorio - KONTRIP VIAGENS.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ23"/>
+  <dimension ref="A1:AQ22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -695,10 +695,10 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
-        <v>22909375</v>
+        <v>23080902</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>23682579</v>
+        <v>23832217</v>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
@@ -706,10 +706,10 @@
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>45911.63607638889</v>
+        <v>45939.81798611111</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>45911.63839120371</v>
+        <v>45939.81917824074</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
@@ -723,7 +723,7 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>HGREKE</t>
+          <t>WCDAHC</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Joaquim Araujo/Antonio</t>
+          <t>Kobo Arruda/Viviane</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="M2" s="6" t="n">
-        <v>45911.50347222222</v>
+        <v>45939.31666666667</v>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
@@ -791,7 +791,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>Cda</t>
+          <t>Total Carnes e Derivados</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -801,11 +801,11 @@
       </c>
       <c r="X2" s="5" t="inlineStr">
         <is>
-          <t>Gol Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y2" s="5" t="n">
-        <v>2145214886</v>
+        <v>2254301906</v>
       </c>
       <c r="Z2" s="5" t="inlineStr">
         <is>
@@ -818,10 +818,10 @@
         </is>
       </c>
       <c r="AB2" s="5" t="n">
-        <v>1054.59</v>
+        <v>1280.28</v>
       </c>
       <c r="AC2" s="5" t="n">
-        <v>51.66</v>
+        <v>450</v>
       </c>
       <c r="AD2" s="5" t="n">
         <v>0</v>
@@ -836,7 +836,7 @@
         <v>0</v>
       </c>
       <c r="AH2" s="5" t="n">
-        <v>94.91</v>
+        <v>40</v>
       </c>
       <c r="AI2" s="5" t="inlineStr">
         <is>
@@ -845,7 +845,7 @@
       </c>
       <c r="AJ2" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 11/09/2025</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 09/10/2025</t>
         </is>
       </c>
       <c r="AK2" s="5" t="inlineStr">
@@ -886,10 +886,10 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>22909351</v>
+        <v>23081304</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>23682559</v>
+        <v>23832603</v>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
@@ -897,10 +897,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>45911.63337962963</v>
+        <v>45939.83322916667</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>45911.63466435186</v>
+        <v>45939.83416666667</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>CONUCR</t>
+          <t>LA9577296IGEK</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>SADER/MARCELO</t>
+          <t>Araujo Sousa/Denival</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="M3" s="6" t="n">
-        <v>45911.50208333333</v>
+        <v>45939.47222222222</v>
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
       </c>
       <c r="V3" s="5" t="inlineStr">
         <is>
-          <t>Cda</t>
+          <t>Perimetral Montagem Ltda</t>
         </is>
       </c>
       <c r="W3" s="5" t="inlineStr">
@@ -992,11 +992,11 @@
       </c>
       <c r="X3" s="5" t="inlineStr">
         <is>
-          <t>Gol Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y3" s="5" t="n">
-        <v>2145214845</v>
+        <v>2254306200</v>
       </c>
       <c r="Z3" s="5" t="inlineStr">
         <is>
@@ -1009,16 +1009,16 @@
         </is>
       </c>
       <c r="AB3" s="5" t="n">
-        <v>2273.89</v>
+        <v>1119.92</v>
       </c>
       <c r="AC3" s="5" t="n">
-        <v>112.28</v>
+        <v>59.46</v>
       </c>
       <c r="AD3" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE3" s="5" t="n">
-        <v>0</v>
+        <v>111.99</v>
       </c>
       <c r="AF3" s="5" t="n">
         <v>0</v>
@@ -1027,7 +1027,7 @@
         <v>0</v>
       </c>
       <c r="AH3" s="5" t="n">
-        <v>204.65</v>
+        <v>73.91</v>
       </c>
       <c r="AI3" s="5" t="inlineStr">
         <is>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="AJ3" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 11/09/2025</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 09/10/2025</t>
         </is>
       </c>
       <c r="AK3" s="5" t="inlineStr">
@@ -1077,10 +1077,10 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>22912227</v>
+        <v>23080569</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>23685269</v>
+        <v>23831910</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -1088,10 +1088,10 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>45911.95170138889</v>
+        <v>45939.794375</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>45911.95275462963</v>
+        <v>45939.79615740741</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>KRJOTN</t>
+          <t>LA9573454KJSA</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Ribeiro/Aldo</t>
+          <t>MOREIRA CAMPOS/RODRIGO</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -1129,7 +1129,7 @@
         </is>
       </c>
       <c r="M4" s="6" t="n">
-        <v>45911.44652777778</v>
+        <v>45939.27430555555</v>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>Pessoa e Pessoa Advogados Associados</t>
+          <t>M3. Business Group Ltda</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="X4" s="5" t="inlineStr">
         <is>
-          <t>Gol Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y4" s="5" t="n">
-        <v>2145247985</v>
+        <v>2254295402</v>
       </c>
       <c r="Z4" s="5" t="inlineStr">
         <is>
@@ -1200,16 +1200,16 @@
         </is>
       </c>
       <c r="AB4" s="5" t="n">
-        <v>489.65</v>
+        <v>1134.32</v>
       </c>
       <c r="AC4" s="5" t="n">
-        <v>44.27</v>
+        <v>49.71</v>
       </c>
       <c r="AD4" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE4" s="5" t="n">
-        <v>0</v>
+        <v>113.43</v>
       </c>
       <c r="AF4" s="5" t="n">
         <v>0</v>
@@ -1218,7 +1218,7 @@
         <v>0</v>
       </c>
       <c r="AH4" s="5" t="n">
-        <v>44.07</v>
+        <v>74.87</v>
       </c>
       <c r="AI4" s="5" t="inlineStr">
         <is>
@@ -1227,7 +1227,7 @@
       </c>
       <c r="AJ4" s="5" t="inlineStr">
         <is>
-          <t>Centro de custo não preenchido! (ACC01)</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 09/10/2025</t>
         </is>
       </c>
       <c r="AK4" s="5" t="inlineStr">
@@ -1237,17 +1237,17 @@
       </c>
       <c r="AL4" s="5" t="inlineStr">
         <is>
-          <t>Centro de custo</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM4" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN4" s="5" t="inlineStr">
         <is>
-          <t>Dados do Fornecedor</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO4" s="5" t="inlineStr">
@@ -1268,10 +1268,10 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>22909965</v>
+        <v>23080570</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>23683184</v>
+        <v>23831911</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
@@ -1279,10 +1279,10 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>45911.70832175926</v>
+        <v>45939.79438657407</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>45911.70954861111</v>
+        <v>45939.79616898148</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
@@ -1296,7 +1296,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>COMIVJ</t>
+          <t>LA9577885KGXX</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>BLENDO FERREIRA SILVA/WILLIAN</t>
+          <t>MOREIRA CAMPOS/RODRIGO</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -1320,7 +1320,7 @@
         </is>
       </c>
       <c r="M5" s="6" t="n">
-        <v>45911.20763888889</v>
+        <v>45939.27430555555</v>
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="V5" s="5" t="inlineStr">
         <is>
-          <t>Rcs Tecnologia S/a</t>
+          <t>M3. Business Group Ltda</t>
         </is>
       </c>
       <c r="W5" s="5" t="inlineStr">
@@ -1374,11 +1374,11 @@
       </c>
       <c r="X5" s="5" t="inlineStr">
         <is>
-          <t>Gol Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y5" s="5" t="n">
-        <v>2145198044</v>
+        <v>2254295499</v>
       </c>
       <c r="Z5" s="5" t="inlineStr">
         <is>
@@ -1391,16 +1391,16 @@
         </is>
       </c>
       <c r="AB5" s="5" t="n">
-        <v>2100.73</v>
+        <v>2799.2</v>
       </c>
       <c r="AC5" s="5" t="n">
-        <v>32.87</v>
+        <v>34.11</v>
       </c>
       <c r="AD5" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE5" s="5" t="n">
-        <v>0</v>
+        <v>279.92</v>
       </c>
       <c r="AF5" s="5" t="n">
         <v>0</v>
@@ -1409,7 +1409,7 @@
         <v>0</v>
       </c>
       <c r="AH5" s="5" t="n">
-        <v>16.67</v>
+        <v>184.75</v>
       </c>
       <c r="AI5" s="5" t="inlineStr">
         <is>
@@ -1418,7 +1418,7 @@
       </c>
       <c r="AJ5" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 11/09/2025</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 09/10/2025</t>
         </is>
       </c>
       <c r="AK5" s="5" t="inlineStr">
@@ -1459,10 +1459,10 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>22910005</v>
+        <v>23079906</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>23683224</v>
+        <v>23831269</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>45911.715625</v>
+        <v>45939.70849537037</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>45911.71751157408</v>
+        <v>45939.70951388889</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>JHVCDE</t>
+          <t>AKPTMJ</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -1497,7 +1497,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>ARAGAO MACEDO/ROGER</t>
+          <t>SILVA/CARLOS</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -1511,7 +1511,7 @@
         </is>
       </c>
       <c r="M6" s="6" t="n">
-        <v>45911.21319444444</v>
+        <v>45939.14722222222</v>
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>Grant Thornton Auditores Independentes</t>
+          <t>M3. Business Group Ltda</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1569,7 +1569,7 @@
         </is>
       </c>
       <c r="Y6" s="5" t="n">
-        <v>2145225407</v>
+        <v>2147053435</v>
       </c>
       <c r="Z6" s="5" t="inlineStr">
         <is>
@@ -1582,10 +1582,10 @@
         </is>
       </c>
       <c r="AB6" s="5" t="n">
-        <v>2966.21</v>
+        <v>687.05</v>
       </c>
       <c r="AC6" s="5" t="n">
-        <v>99.81999999999999</v>
+        <v>51.67</v>
       </c>
       <c r="AD6" s="5" t="n">
         <v>0</v>
@@ -1600,7 +1600,7 @@
         <v>0</v>
       </c>
       <c r="AH6" s="5" t="n">
-        <v>156.11</v>
+        <v>68.70999999999999</v>
       </c>
       <c r="AI6" s="5" t="inlineStr">
         <is>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="AJ6" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 11/09/2025</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 09/10/2025</t>
         </is>
       </c>
       <c r="AK6" s="5" t="inlineStr">
@@ -1650,10 +1650,10 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>22909453</v>
+        <v>23080330</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>23682661</v>
+        <v>23831677</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
@@ -1661,10 +1661,10 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>45911.64583333334</v>
+        <v>45939.75549768518</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>45911.64748842592</v>
+        <v>45939.75674768518</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
@@ -1678,7 +1678,7 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>DKPNID</t>
+          <t>XGRVNY</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Schwind/Luís</t>
+          <t>leal/maria</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -1702,7 +1702,7 @@
         </is>
       </c>
       <c r="M7" s="6" t="n">
-        <v>45911.12013888889</v>
+        <v>45939.2375</v>
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="V7" s="5" t="inlineStr">
         <is>
-          <t>Basso e Pancotte Ltda</t>
+          <t>M3. Business Group Ltda</t>
         </is>
       </c>
       <c r="W7" s="5" t="inlineStr">
@@ -1756,11 +1756,11 @@
       </c>
       <c r="X7" s="5" t="inlineStr">
         <is>
-          <t>Gol Linhas Aereas</t>
+          <t>Azul Linhas Aereas</t>
         </is>
       </c>
       <c r="Y7" s="5" t="n">
-        <v>660876</v>
+        <v>692643443</v>
       </c>
       <c r="Z7" s="5" t="inlineStr">
         <is>
@@ -1773,10 +1773,10 @@
         </is>
       </c>
       <c r="AB7" s="5" t="n">
-        <v>637.14</v>
+        <v>408.67</v>
       </c>
       <c r="AC7" s="5" t="n">
-        <v>47.02</v>
+        <v>34.11</v>
       </c>
       <c r="AD7" s="5" t="n">
         <v>0</v>
@@ -1791,7 +1791,7 @@
         <v>0</v>
       </c>
       <c r="AH7" s="5" t="n">
-        <v>229.37</v>
+        <v>20.43</v>
       </c>
       <c r="AI7" s="5" t="inlineStr">
         <is>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="AJ7" s="5" t="inlineStr">
         <is>
-          <t>Verificação de bilhetes: Bilhete 660876 já sendo utilizado para este fornecedor.</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 09/10/2025</t>
         </is>
       </c>
       <c r="AK7" s="5" t="inlineStr">
@@ -1810,17 +1810,17 @@
       </c>
       <c r="AL7" s="5" t="inlineStr">
         <is>
-          <t>Bilhete duplicado</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM7" s="5" t="inlineStr">
         <is>
-          <t>Bilhete Já Contabilizado</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN7" s="5" t="inlineStr">
         <is>
-          <t>Duplicidade de Contabilização</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO7" s="5" t="inlineStr">
@@ -1841,21 +1841,21 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
-        <v>22909453</v>
+        <v>23077346</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>23682662</v>
+        <v>23828750</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>ACC02</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>45911.64583333334</v>
+        <v>45939.45822916667</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>45911.64748842592</v>
+        <v>45939.45974537037</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
@@ -1869,7 +1869,7 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>DKPNID</t>
+          <t>yagnqp</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -1879,7 +1879,7 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Bonvini/Bianca</t>
+          <t>DA ROCHA ZANOT/ALESSANDRA</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1893,7 +1893,7 @@
         </is>
       </c>
       <c r="M8" s="6" t="n">
-        <v>45911.12013888889</v>
+        <v>45939.45694444444</v>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>Basso e Pancotte Ltda</t>
+          <t>Grant Thornton Auditores Independentes</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1951,7 +1951,7 @@
         </is>
       </c>
       <c r="Y8" s="5" t="n">
-        <v>660876</v>
+        <v>2147022229</v>
       </c>
       <c r="Z8" s="5" t="inlineStr">
         <is>
@@ -1964,10 +1964,10 @@
         </is>
       </c>
       <c r="AB8" s="5" t="n">
-        <v>637.14</v>
+        <v>1413.07</v>
       </c>
       <c r="AC8" s="5" t="n">
-        <v>47.02</v>
+        <v>0</v>
       </c>
       <c r="AD8" s="5" t="n">
         <v>0</v>
@@ -1982,7 +1982,7 @@
         <v>0</v>
       </c>
       <c r="AH8" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="AI8" s="5" t="inlineStr">
         <is>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="AJ8" s="5" t="inlineStr">
         <is>
-          <t>Verificação de bilhetes: Bilhete 660876 já sendo utilizado para este fornecedor.</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 09/10/2025</t>
         </is>
       </c>
       <c r="AK8" s="5" t="inlineStr">
@@ -2001,17 +2001,17 @@
       </c>
       <c r="AL8" s="5" t="inlineStr">
         <is>
-          <t>Bilhete duplicado</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM8" s="5" t="inlineStr">
         <is>
-          <t>Bilhete Já Contabilizado</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN8" s="5" t="inlineStr">
         <is>
-          <t>Duplicidade de Contabilização</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO8" s="5" t="inlineStr">
@@ -2032,21 +2032,21 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>22909453</v>
+        <v>23077563</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>23682663</v>
+        <v>23828950</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>ACC03</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>45911.64583333334</v>
+        <v>45939.48603009259</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>45911.64748842592</v>
+        <v>45939.48840277778</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
@@ -2060,7 +2060,7 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>DKPNID</t>
+          <t>LA9576070TAXM</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Harami/Priscila</t>
+          <t>REZENDE/IRAM</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
@@ -2084,7 +2084,7 @@
         </is>
       </c>
       <c r="M9" s="6" t="n">
-        <v>45911.12013888889</v>
+        <v>45939.46736111111</v>
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="V9" s="5" t="inlineStr">
         <is>
-          <t>Basso e Pancotte Ltda</t>
+          <t>M3. Business Group Ltda</t>
         </is>
       </c>
       <c r="W9" s="5" t="inlineStr">
@@ -2138,11 +2138,11 @@
       </c>
       <c r="X9" s="5" t="inlineStr">
         <is>
-          <t>Gol Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y9" s="5" t="n">
-        <v>660876</v>
+        <v>2254211035</v>
       </c>
       <c r="Z9" s="5" t="inlineStr">
         <is>
@@ -2155,16 +2155,16 @@
         </is>
       </c>
       <c r="AB9" s="5" t="n">
-        <v>637.14</v>
+        <v>2171.12</v>
       </c>
       <c r="AC9" s="5" t="n">
-        <v>47.02</v>
+        <v>32.87</v>
       </c>
       <c r="AD9" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE9" s="5" t="n">
-        <v>0</v>
+        <v>217.11</v>
       </c>
       <c r="AF9" s="5" t="n">
         <v>0</v>
@@ -2173,7 +2173,7 @@
         <v>0</v>
       </c>
       <c r="AH9" s="5" t="n">
-        <v>0</v>
+        <v>143.29</v>
       </c>
       <c r="AI9" s="5" t="inlineStr">
         <is>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="AJ9" s="5" t="inlineStr">
         <is>
-          <t>Verificação de bilhetes: Bilhete 660876 já sendo utilizado para este fornecedor.</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 09/10/2025</t>
         </is>
       </c>
       <c r="AK9" s="5" t="inlineStr">
@@ -2192,17 +2192,17 @@
       </c>
       <c r="AL9" s="5" t="inlineStr">
         <is>
-          <t>Bilhete duplicado</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM9" s="5" t="inlineStr">
         <is>
-          <t>Bilhete Já Contabilizado</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN9" s="5" t="inlineStr">
         <is>
-          <t>Duplicidade de Contabilização</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO9" s="5" t="inlineStr">
@@ -2223,21 +2223,21 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>22909453</v>
+        <v>23077512</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>23682664</v>
+        <v>23828905</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>ACC04</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>45911.64583333334</v>
+        <v>45939.47908564815</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>45911.64748842592</v>
+        <v>45939.48043981481</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>DKPNID</t>
+          <t>UL7QKZ</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Schwind/Amanda</t>
+          <t>GUIMARAES/GUSTAVO</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -2275,7 +2275,7 @@
         </is>
       </c>
       <c r="M10" s="6" t="n">
-        <v>45911.12013888889</v>
+        <v>45939.45138888889</v>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>Basso e Pancotte Ltda</t>
+          <t>M3. Business Group Ltda</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -2329,11 +2329,11 @@
       </c>
       <c r="X10" s="5" t="inlineStr">
         <is>
-          <t>Gol Linhas Aereas</t>
+          <t>Azul Linhas Aereas</t>
         </is>
       </c>
       <c r="Y10" s="5" t="n">
-        <v>827692</v>
+        <v>860843023</v>
       </c>
       <c r="Z10" s="5" t="inlineStr">
         <is>
@@ -2346,10 +2346,10 @@
         </is>
       </c>
       <c r="AB10" s="5" t="n">
-        <v>637.14</v>
+        <v>749.17</v>
       </c>
       <c r="AC10" s="5" t="n">
-        <v>47.02</v>
+        <v>33.56</v>
       </c>
       <c r="AD10" s="5" t="n">
         <v>0</v>
@@ -2364,7 +2364,7 @@
         <v>0</v>
       </c>
       <c r="AH10" s="5" t="n">
-        <v>0</v>
+        <v>37.46</v>
       </c>
       <c r="AI10" s="5" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
       </c>
       <c r="AJ10" s="5" t="inlineStr">
         <is>
-          <t>Verificação de bilhetes: Bilhete 660876 já sendo utilizado para este fornecedor.</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 09/10/2025</t>
         </is>
       </c>
       <c r="AK10" s="5" t="inlineStr">
@@ -2383,17 +2383,17 @@
       </c>
       <c r="AL10" s="5" t="inlineStr">
         <is>
-          <t>Bilhete duplicado</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM10" s="5" t="inlineStr">
         <is>
-          <t>Bilhete Já Contabilizado</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN10" s="5" t="inlineStr">
         <is>
-          <t>Duplicidade de Contabilização</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO10" s="5" t="inlineStr">
@@ -2414,10 +2414,10 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
-        <v>22861685</v>
+        <v>23079151</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>23641631</v>
+        <v>23830527</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
@@ -2425,24 +2425,24 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>45903.61025462963</v>
+        <v>45939.61383101852</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>45903.61174768519</v>
+        <v>45939.61511574074</v>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>CCIMEA</t>
+          <t>VQSWTX</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
@@ -2452,7 +2452,7 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>Venceslau dos Santos/Alisson</t>
+          <t>POLTRONIERI/MARCELLO</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
@@ -2466,7 +2466,7 @@
         </is>
       </c>
       <c r="M11" s="6" t="n">
-        <v>45903.51736111111</v>
+        <v>45939.11319444444</v>
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
@@ -2505,12 +2505,12 @@
       </c>
       <c r="U11" s="5" t="inlineStr">
         <is>
-          <t>Grupo Mercurio York</t>
+          <t>Grupo Kontrip</t>
         </is>
       </c>
       <c r="V11" s="5" t="inlineStr">
         <is>
-          <t>Agencia Mercurio York Viagens e Turismo Ltda</t>
+          <t>Cinesystem S.a.</t>
         </is>
       </c>
       <c r="W11" s="5" t="inlineStr">
@@ -2520,11 +2520,11 @@
       </c>
       <c r="X11" s="5" t="inlineStr">
         <is>
-          <t>Gol Linhas Aereas</t>
+          <t>Azul Linhas Aereas</t>
         </is>
       </c>
       <c r="Y11" s="5" t="n">
-        <v>2144712008</v>
+        <v>546952371</v>
       </c>
       <c r="Z11" s="5" t="inlineStr">
         <is>
@@ -2537,10 +2537,10 @@
         </is>
       </c>
       <c r="AB11" s="5" t="n">
-        <v>1483.11</v>
+        <v>1002.75</v>
       </c>
       <c r="AC11" s="5" t="n">
-        <v>44.27</v>
+        <v>450</v>
       </c>
       <c r="AD11" s="5" t="n">
         <v>0</v>
@@ -2555,7 +2555,7 @@
         <v>0</v>
       </c>
       <c r="AH11" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="AI11" s="5" t="inlineStr">
         <is>
@@ -2564,7 +2564,7 @@
       </c>
       <c r="AJ11" s="5" t="inlineStr">
         <is>
-          <t>Centro de custo não preenchido! (ACC01)</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 09/10/2025</t>
         </is>
       </c>
       <c r="AK11" s="5" t="inlineStr">
@@ -2574,17 +2574,17 @@
       </c>
       <c r="AL11" s="5" t="inlineStr">
         <is>
-          <t>Centro de custo</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM11" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN11" s="5" t="inlineStr">
         <is>
-          <t>Dados do Fornecedor</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO11" s="5" t="inlineStr">
@@ -2605,10 +2605,10 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
-        <v>22861689</v>
+        <v>23079979</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>23641636</v>
+        <v>23831337</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
@@ -2616,24 +2616,24 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>45903.61160879629</v>
+        <v>45939.71254629629</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>45903.61373842593</v>
+        <v>45939.71363425926</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>CVENDX</t>
+          <t>DLKNNG</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Vilela/Lidiany</t>
+          <t>DAMASCENO/ABRAAO</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -2657,7 +2657,7 @@
         </is>
       </c>
       <c r="M12" s="6" t="n">
-        <v>45903.51527777778</v>
+        <v>45939.19652777778</v>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
@@ -2696,12 +2696,12 @@
       </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>Grupo Mercurio York</t>
+          <t>Grupo Kontrip</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>Agencia Mercurio York Viagens e Turismo Ltda</t>
+          <t>M3. Business Group Ltda</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -2711,11 +2711,11 @@
       </c>
       <c r="X12" s="5" t="inlineStr">
         <is>
-          <t>Gol Linhas Aereas</t>
+          <t>Azul Linhas Aereas</t>
         </is>
       </c>
       <c r="Y12" s="5" t="n">
-        <v>2144711372</v>
+        <v>998521164</v>
       </c>
       <c r="Z12" s="5" t="inlineStr">
         <is>
@@ -2728,10 +2728,10 @@
         </is>
       </c>
       <c r="AB12" s="5" t="n">
-        <v>954.8099999999999</v>
+        <v>2653.15</v>
       </c>
       <c r="AC12" s="5" t="n">
-        <v>44.27</v>
+        <v>96.13</v>
       </c>
       <c r="AD12" s="5" t="n">
         <v>0</v>
@@ -2746,7 +2746,7 @@
         <v>0</v>
       </c>
       <c r="AH12" s="5" t="n">
-        <v>0</v>
+        <v>132.66</v>
       </c>
       <c r="AI12" s="5" t="inlineStr">
         <is>
@@ -2755,7 +2755,7 @@
       </c>
       <c r="AJ12" s="5" t="inlineStr">
         <is>
-          <t>Centro de custo não preenchido! (ACC01)</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 09/10/2025</t>
         </is>
       </c>
       <c r="AK12" s="5" t="inlineStr">
@@ -2765,17 +2765,17 @@
       </c>
       <c r="AL12" s="5" t="inlineStr">
         <is>
-          <t>Centro de custo</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM12" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN12" s="5" t="inlineStr">
         <is>
-          <t>Dados do Fornecedor</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO12" s="5" t="inlineStr">
@@ -2796,10 +2796,10 @@
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
-        <v>22862473</v>
+        <v>23078240</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>23642350</v>
+        <v>23829621</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
@@ -2807,24 +2807,24 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>45903.72704861111</v>
+        <v>45939.56243055555</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>45903.72773148148</v>
+        <v>45939.56340277778</v>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>HRLZLB</t>
+          <t>EUEPYS</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>ANGE ARAUJO/ENY</t>
+          <t>ANTONIO DA SILVA SANTOS LIMA/MARCO</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
@@ -2848,7 +2848,7 @@
         </is>
       </c>
       <c r="M13" s="6" t="n">
-        <v>45903.20902777778</v>
+        <v>45939.06180555555</v>
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
@@ -2887,12 +2887,12 @@
       </c>
       <c r="U13" s="5" t="inlineStr">
         <is>
-          <t>Grupo Mercurio York</t>
+          <t>Grupo Kontrip</t>
         </is>
       </c>
       <c r="V13" s="5" t="inlineStr">
         <is>
-          <t>Agencia Mercurio York Viagens e Turismo Ltda</t>
+          <t>Broadtec Tecnologia e Servicos Ltda</t>
         </is>
       </c>
       <c r="W13" s="5" t="inlineStr">
@@ -2906,7 +2906,7 @@
         </is>
       </c>
       <c r="Y13" s="5" t="n">
-        <v>2144726580</v>
+        <v>2146905230</v>
       </c>
       <c r="Z13" s="5" t="inlineStr">
         <is>
@@ -2919,10 +2919,10 @@
         </is>
       </c>
       <c r="AB13" s="5" t="n">
-        <v>539.01</v>
+        <v>545.96</v>
       </c>
       <c r="AC13" s="5" t="n">
-        <v>60.62</v>
+        <v>878.22</v>
       </c>
       <c r="AD13" s="5" t="n">
         <v>0</v>
@@ -2937,7 +2937,7 @@
         <v>0</v>
       </c>
       <c r="AH13" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="AI13" s="5" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       </c>
       <c r="AJ13" s="5" t="inlineStr">
         <is>
-          <t>Centro de custo não preenchido! (ACC02)</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 09/10/2025</t>
         </is>
       </c>
       <c r="AK13" s="5" t="inlineStr">
@@ -2956,17 +2956,17 @@
       </c>
       <c r="AL13" s="5" t="inlineStr">
         <is>
-          <t>Centro de custo</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM13" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN13" s="5" t="inlineStr">
         <is>
-          <t>Dados do Fornecedor</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO13" s="5" t="inlineStr">
@@ -2987,35 +2987,35 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
-        <v>22862473</v>
+        <v>23078383</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>23642351</v>
+        <v>23829756</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>ACC02</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>45903.72704861111</v>
+        <v>45939.56799768518</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>45903.72773148148</v>
+        <v>45939.56938657408</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>HRLZLB</t>
+          <t>JRUOAE</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
@@ -3025,7 +3025,7 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>OLIVEIRA/PRISCILA</t>
+          <t>MENEZES DA SILVA/ROBSON</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -3039,7 +3039,7 @@
         </is>
       </c>
       <c r="M14" s="6" t="n">
-        <v>45903.20902777778</v>
+        <v>45939.06666666667</v>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
@@ -3078,12 +3078,12 @@
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>Grupo Mercurio York</t>
+          <t>Grupo Kontrip</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
         <is>
-          <t>Agencia Mercurio York Viagens e Turismo Ltda</t>
+          <t>Broadtec Tecnologia e Servicos Ltda</t>
         </is>
       </c>
       <c r="W14" s="5" t="inlineStr">
@@ -3097,7 +3097,7 @@
         </is>
       </c>
       <c r="Y14" s="5" t="n">
-        <v>2144726581</v>
+        <v>2146895657</v>
       </c>
       <c r="Z14" s="5" t="inlineStr">
         <is>
@@ -3110,10 +3110,10 @@
         </is>
       </c>
       <c r="AB14" s="5" t="n">
-        <v>539.01</v>
+        <v>545.96</v>
       </c>
       <c r="AC14" s="5" t="n">
-        <v>60.62</v>
+        <v>878.22</v>
       </c>
       <c r="AD14" s="5" t="n">
         <v>0</v>
@@ -3128,7 +3128,7 @@
         <v>0</v>
       </c>
       <c r="AH14" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="AI14" s="5" t="inlineStr">
         <is>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="AJ14" s="5" t="inlineStr">
         <is>
-          <t>Centro de custo não preenchido! (ACC02)</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 09/10/2025</t>
         </is>
       </c>
       <c r="AK14" s="5" t="inlineStr">
@@ -3147,17 +3147,17 @@
       </c>
       <c r="AL14" s="5" t="inlineStr">
         <is>
-          <t>Centro de custo</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM14" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN14" s="5" t="inlineStr">
         <is>
-          <t>Dados do Fornecedor</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO14" s="5" t="inlineStr">
@@ -3178,10 +3178,10 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
-        <v>22874109</v>
+        <v>23077812</v>
       </c>
       <c r="B15" s="5" t="n">
-        <v>23652657</v>
+        <v>23829194</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
@@ -3189,24 +3189,24 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>45905.4492824074</v>
+        <v>45939.52912037037</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>45905.45436342592</v>
+        <v>45939.52975694444</v>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>LA9575496KNXE</t>
+          <t>TM3IPW</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>Rios/Aline</t>
+          <t>Alcântara/Pedro</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
@@ -3230,7 +3230,7 @@
         </is>
       </c>
       <c r="M15" s="6" t="n">
-        <v>45905.44166666667</v>
+        <v>45939.46527777778</v>
       </c>
       <c r="N15" s="5" t="inlineStr">
         <is>
@@ -3269,12 +3269,12 @@
       </c>
       <c r="U15" s="5" t="inlineStr">
         <is>
-          <t>Grupo Mercurio York</t>
+          <t>Grupo Kontrip</t>
         </is>
       </c>
       <c r="V15" s="5" t="inlineStr">
         <is>
-          <t>Agencia Mercurio York Viagens e Turismo Ltda</t>
+          <t>Viva Studio Oral</t>
         </is>
       </c>
       <c r="W15" s="5" t="inlineStr">
@@ -3284,11 +3284,11 @@
       </c>
       <c r="X15" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Azul Linhas Aereas</t>
         </is>
       </c>
       <c r="Y15" s="5" t="n">
-        <v>2249116391</v>
+        <v>605774081</v>
       </c>
       <c r="Z15" s="5" t="inlineStr">
         <is>
@@ -3301,10 +3301,10 @@
         </is>
       </c>
       <c r="AB15" s="5" t="n">
-        <v>1873.44</v>
+        <v>863.58</v>
       </c>
       <c r="AC15" s="5" t="n">
-        <v>77.14</v>
+        <v>99.97</v>
       </c>
       <c r="AD15" s="5" t="n">
         <v>0</v>
@@ -3319,7 +3319,7 @@
         <v>0</v>
       </c>
       <c r="AH15" s="5" t="n">
-        <v>0</v>
+        <v>103.63</v>
       </c>
       <c r="AI15" s="5" t="inlineStr">
         <is>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="AJ15" s="5" t="inlineStr">
         <is>
-          <t>Centro de custo não preenchido! (ACC02)</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 09/10/2025</t>
         </is>
       </c>
       <c r="AK15" s="5" t="inlineStr">
@@ -3338,17 +3338,17 @@
       </c>
       <c r="AL15" s="5" t="inlineStr">
         <is>
-          <t>Centro de custo</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM15" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN15" s="5" t="inlineStr">
         <is>
-          <t>Dados do Fornecedor</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO15" s="5" t="inlineStr">
@@ -3369,35 +3369,35 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
-        <v>22874109</v>
+        <v>23079350</v>
       </c>
       <c r="B16" s="5" t="n">
-        <v>23652659</v>
+        <v>23830724</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>ACC02</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D16" s="6" t="n">
-        <v>45905.4492824074</v>
+        <v>45939.63207175926</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>45905.45436342592</v>
+        <v>45939.63369212963</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>LA9575496KNXE</t>
+          <t>MRNXIL</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
@@ -3407,7 +3407,7 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Luz Santos/Uendeo</t>
+          <t>botelho/roberto</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -3421,7 +3421,7 @@
         </is>
       </c>
       <c r="M16" s="6" t="n">
-        <v>45905.44166666667</v>
+        <v>45939.10902777778</v>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
@@ -3460,12 +3460,12 @@
       </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>Grupo Mercurio York</t>
+          <t>Grupo Kontrip</t>
         </is>
       </c>
       <c r="V16" s="5" t="inlineStr">
         <is>
-          <t>Agencia Mercurio York Viagens e Turismo Ltda</t>
+          <t>Daten Tecnologia</t>
         </is>
       </c>
       <c r="W16" s="5" t="inlineStr">
@@ -3479,7 +3479,7 @@
         </is>
       </c>
       <c r="Y16" s="5" t="n">
-        <v>2249116392</v>
+        <v>2254242120</v>
       </c>
       <c r="Z16" s="5" t="inlineStr">
         <is>
@@ -3492,10 +3492,10 @@
         </is>
       </c>
       <c r="AB16" s="5" t="n">
-        <v>1873.44</v>
+        <v>0.01</v>
       </c>
       <c r="AC16" s="5" t="n">
-        <v>77.14</v>
+        <v>0</v>
       </c>
       <c r="AD16" s="5" t="n">
         <v>0</v>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="AJ16" s="5" t="inlineStr">
         <is>
-          <t>Centro de custo não preenchido! (ACC02)</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 09/10/2025</t>
         </is>
       </c>
       <c r="AK16" s="5" t="inlineStr">
@@ -3529,17 +3529,17 @@
       </c>
       <c r="AL16" s="5" t="inlineStr">
         <is>
-          <t>Centro de custo</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM16" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN16" s="5" t="inlineStr">
         <is>
-          <t>Dados do Fornecedor</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO16" s="5" t="inlineStr">
@@ -3560,21 +3560,21 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
-        <v>22911619</v>
+        <v>23079146</v>
       </c>
       <c r="B17" s="5" t="n">
-        <v>23684774</v>
+        <v>23830533</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>ACC01</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="D17" s="6" t="n">
-        <v>45911.82673611111</v>
+        <v>45939.61219907407</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>45911.82756944445</v>
+        <v>45939.61859953704</v>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
@@ -3588,31 +3588,31 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>LA9571454MECM</t>
+          <t>TQH66H</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>EBOOKING</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>Ribeiro Marques Moura/Adriana</t>
+          <t>JEAN GOMES DA SILVA</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>Kontrip</t>
+          <t>Juliana Cardoso</t>
         </is>
       </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
-          <t>Kontrip</t>
+          <t>Juliana Cardoso</t>
         </is>
       </c>
       <c r="M17" s="6" t="n">
-        <v>45911.31458333333</v>
+        <v>45938.61180555556</v>
       </c>
       <c r="N17" s="5" t="inlineStr">
         <is>
@@ -3656,7 +3656,7 @@
       </c>
       <c r="V17" s="5" t="inlineStr">
         <is>
-          <t>Grant Thornton Auditores Independentes</t>
+          <t>Kontrip - Vendas Cartao de Credito</t>
         </is>
       </c>
       <c r="W17" s="5" t="inlineStr">
@@ -3666,11 +3666,11 @@
       </c>
       <c r="X17" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Azul Linhas Aereas</t>
         </is>
       </c>
       <c r="Y17" s="5" t="n">
-        <v>2250076385</v>
+        <v>3023830532</v>
       </c>
       <c r="Z17" s="5" t="inlineStr">
         <is>
@@ -3683,16 +3683,16 @@
         </is>
       </c>
       <c r="AB17" s="5" t="n">
-        <v>823.84</v>
+        <v>2202.12</v>
       </c>
       <c r="AC17" s="5" t="n">
-        <v>120.57</v>
+        <v>46.36</v>
       </c>
       <c r="AD17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE17" s="5" t="n">
-        <v>82.38</v>
+        <v>0</v>
       </c>
       <c r="AF17" s="5" t="n">
         <v>0</v>
@@ -3701,16 +3701,16 @@
         <v>0</v>
       </c>
       <c r="AH17" s="5" t="n">
-        <v>36.25</v>
+        <v>264.25</v>
       </c>
       <c r="AI17" s="5" t="inlineStr">
         <is>
-          <t>obs</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AJ17" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 11/09/2025</t>
+          <t xml:space="preserve">35Ocorreu a seguinte exceção ao gerar a ordem de venda: Ocorreu a seguinte exceção ao inserir o item da ordem de venda:  Faltou informar rateio de </t>
         </is>
       </c>
       <c r="AK17" s="5" t="inlineStr">
@@ -3720,17 +3720,17 @@
       </c>
       <c r="AL17" s="5" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>Falta de informação Gerencial</t>
         </is>
       </c>
       <c r="AM17" s="5" t="inlineStr">
         <is>
-          <t>Análise Benner</t>
+          <t>Rateio de centro de custo/projeto</t>
         </is>
       </c>
       <c r="AN17" s="5" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Dados Gerenciais</t>
         </is>
       </c>
       <c r="AO17" s="5" t="inlineStr">
@@ -3751,10 +3751,10 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
-        <v>22908935</v>
+        <v>23078778</v>
       </c>
       <c r="B18" s="5" t="n">
-        <v>23682176</v>
+        <v>23830152</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
@@ -3762,10 +3762,10 @@
         </is>
       </c>
       <c r="D18" s="6" t="n">
-        <v>45911.5708912037</v>
+        <v>45939.5825</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>45911.57164351852</v>
+        <v>45939.58415509259</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
@@ -3779,7 +3779,7 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>UBVDEP</t>
+          <t>FSYKDL</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>RODRIGUES MAUES ALVES/DEBORA</t>
+          <t>Dias/Eloa</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -3803,7 +3803,7 @@
         </is>
       </c>
       <c r="M18" s="6" t="n">
-        <v>45911.06944444445</v>
+        <v>45939.07847222222</v>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
@@ -3842,12 +3842,12 @@
       </c>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>Grupo Kontrip</t>
+          <t>Grupo Mercurio York</t>
         </is>
       </c>
       <c r="V18" s="5" t="inlineStr">
         <is>
-          <t>Mobiauto Edicao de Anuncios On Line Ltda</t>
+          <t>Agencia Mercurio York Viagens e Turismo Ltda</t>
         </is>
       </c>
       <c r="W18" s="5" t="inlineStr">
@@ -3857,11 +3857,11 @@
       </c>
       <c r="X18" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Gol Linhas Aereas</t>
         </is>
       </c>
       <c r="Y18" s="5" t="n">
-        <v>2250011889</v>
+        <v>2147036576</v>
       </c>
       <c r="Z18" s="5" t="inlineStr">
         <is>
@@ -3874,10 +3874,10 @@
         </is>
       </c>
       <c r="AB18" s="5" t="n">
-        <v>258</v>
+        <v>3759.86</v>
       </c>
       <c r="AC18" s="5" t="n">
-        <v>450</v>
+        <v>113.34</v>
       </c>
       <c r="AD18" s="5" t="n">
         <v>0</v>
@@ -3892,7 +3892,7 @@
         <v>0</v>
       </c>
       <c r="AH18" s="5" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="AI18" s="5" t="inlineStr">
         <is>
@@ -3901,7 +3901,7 @@
       </c>
       <c r="AJ18" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 11/09/2025</t>
+          <t>Centro de custo não preenchido! (ACC01)</t>
         </is>
       </c>
       <c r="AK18" s="5" t="inlineStr">
@@ -3911,17 +3911,17 @@
       </c>
       <c r="AL18" s="5" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>Centro de custo</t>
         </is>
       </c>
       <c r="AM18" s="5" t="inlineStr">
         <is>
-          <t>Análise Benner</t>
+          <t>Falta de informação Gerencial</t>
         </is>
       </c>
       <c r="AN18" s="5" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Dados do Fornecedor</t>
         </is>
       </c>
       <c r="AO18" s="5" t="inlineStr">
@@ -3942,10 +3942,10 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>22909200</v>
+        <v>23078887</v>
       </c>
       <c r="B19" s="5" t="n">
-        <v>23682403</v>
+        <v>23830258</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
@@ -3953,10 +3953,10 @@
         </is>
       </c>
       <c r="D19" s="6" t="n">
-        <v>45911.61798611111</v>
+        <v>45939.58658564815</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>45911.61986111111</v>
+        <v>45939.58788194445</v>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
@@ -3970,7 +3970,7 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>LA9574225TCIL</t>
+          <t>IDDCOZ</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
@@ -3980,7 +3980,7 @@
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>Vasconcelos/Maíra</t>
+          <t>Mota/Luiza</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
@@ -3994,7 +3994,7 @@
         </is>
       </c>
       <c r="M19" s="6" t="n">
-        <v>45910.44583333333</v>
+        <v>45939.08194444444</v>
       </c>
       <c r="N19" s="5" t="inlineStr">
         <is>
@@ -4033,12 +4033,12 @@
       </c>
       <c r="U19" s="5" t="inlineStr">
         <is>
-          <t>Grupo Kontrip</t>
+          <t>Grupo Mercurio York</t>
         </is>
       </c>
       <c r="V19" s="5" t="inlineStr">
         <is>
-          <t>Mega Logistica Transporte Por Navegacao S/a</t>
+          <t>Agencia Mercurio York Viagens e Turismo Ltda</t>
         </is>
       </c>
       <c r="W19" s="5" t="inlineStr">
@@ -4048,11 +4048,11 @@
       </c>
       <c r="X19" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Gol Linhas Aereas</t>
         </is>
       </c>
       <c r="Y19" s="5" t="n">
-        <v>2250024175</v>
+        <v>2147037099</v>
       </c>
       <c r="Z19" s="5" t="inlineStr">
         <is>
@@ -4065,16 +4065,16 @@
         </is>
       </c>
       <c r="AB19" s="5" t="n">
-        <v>1894.32</v>
+        <v>1912.28</v>
       </c>
       <c r="AC19" s="5" t="n">
-        <v>33.64</v>
+        <v>52.72</v>
       </c>
       <c r="AD19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE19" s="5" t="n">
-        <v>189.43</v>
+        <v>0</v>
       </c>
       <c r="AF19" s="5" t="n">
         <v>0</v>
@@ -4083,7 +4083,7 @@
         <v>0</v>
       </c>
       <c r="AH19" s="5" t="n">
-        <v>250.05</v>
+        <v>0</v>
       </c>
       <c r="AI19" s="5" t="inlineStr">
         <is>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="AJ19" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 10/09/2025</t>
+          <t>Centro de custo não preenchido! (ACC01)</t>
         </is>
       </c>
       <c r="AK19" s="5" t="inlineStr">
@@ -4102,17 +4102,17 @@
       </c>
       <c r="AL19" s="5" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>Centro de custo</t>
         </is>
       </c>
       <c r="AM19" s="5" t="inlineStr">
         <is>
-          <t>Análise Benner</t>
+          <t>Falta de informação Gerencial</t>
         </is>
       </c>
       <c r="AN19" s="5" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Dados do Fornecedor</t>
         </is>
       </c>
       <c r="AO19" s="5" t="inlineStr">
@@ -4133,21 +4133,21 @@
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
-        <v>22909200</v>
+        <v>23069422</v>
       </c>
       <c r="B20" s="5" t="n">
-        <v>23682404</v>
+        <v>23821363</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>ACC02</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>45911.61798611111</v>
+        <v>45938.42263888889</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>45911.61986111111</v>
+        <v>45938.4233912037</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
@@ -4161,7 +4161,7 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>LA9574225TCIL</t>
+          <t>AVZBXY</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
@@ -4171,7 +4171,7 @@
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>Carvalho/Eduardo</t>
+          <t>BARRETO/LUCIANA</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
@@ -4185,7 +4185,7 @@
         </is>
       </c>
       <c r="M20" s="6" t="n">
-        <v>45910.44583333333</v>
+        <v>45938.41805555556</v>
       </c>
       <c r="N20" s="5" t="inlineStr">
         <is>
@@ -4224,12 +4224,12 @@
       </c>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>Grupo Kontrip</t>
+          <t>Grupo Mercurio York</t>
         </is>
       </c>
       <c r="V20" s="5" t="inlineStr">
         <is>
-          <t>Mega Logistica Transporte Por Navegacao S/a</t>
+          <t>Agencia Mercurio York Viagens e Turismo Ltda</t>
         </is>
       </c>
       <c r="W20" s="5" t="inlineStr">
@@ -4239,11 +4239,11 @@
       </c>
       <c r="X20" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Gol Linhas Aereas</t>
         </is>
       </c>
       <c r="Y20" s="5" t="n">
-        <v>2250024176</v>
+        <v>2146940840</v>
       </c>
       <c r="Z20" s="5" t="inlineStr">
         <is>
@@ -4256,16 +4256,16 @@
         </is>
       </c>
       <c r="AB20" s="5" t="n">
-        <v>1894.32</v>
+        <v>512.61</v>
       </c>
       <c r="AC20" s="5" t="n">
-        <v>33.64</v>
+        <v>49.71</v>
       </c>
       <c r="AD20" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE20" s="5" t="n">
-        <v>189.43</v>
+        <v>0</v>
       </c>
       <c r="AF20" s="5" t="n">
         <v>0</v>
@@ -4283,7 +4283,7 @@
       </c>
       <c r="AJ20" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 10/09/2025</t>
+          <t>Centro de custo não preenchido! (ACC01)</t>
         </is>
       </c>
       <c r="AK20" s="5" t="inlineStr">
@@ -4293,17 +4293,17 @@
       </c>
       <c r="AL20" s="5" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>Centro de custo</t>
         </is>
       </c>
       <c r="AM20" s="5" t="inlineStr">
         <is>
-          <t>Análise Benner</t>
+          <t>Falta de informação Gerencial</t>
         </is>
       </c>
       <c r="AN20" s="5" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Dados do Fornecedor</t>
         </is>
       </c>
       <c r="AO20" s="5" t="inlineStr">
@@ -4324,10 +4324,10 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
-        <v>22909804</v>
+        <v>23069453</v>
       </c>
       <c r="B21" s="5" t="n">
-        <v>23683039</v>
+        <v>23821404</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
@@ -4335,10 +4335,10 @@
         </is>
       </c>
       <c r="D21" s="6" t="n">
-        <v>45911.69021990741</v>
+        <v>45938.42708333334</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>45911.6922337963</v>
+        <v>45938.42769675926</v>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
@@ -4352,7 +4352,7 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>LA9573321XRQH</t>
+          <t>LH164F</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>SILVA/DANIEL</t>
+          <t>BARRETO/LUCIANA</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
@@ -4376,7 +4376,7 @@
         </is>
       </c>
       <c r="M21" s="6" t="n">
-        <v>45911.42777777778</v>
+        <v>45938.42222222222</v>
       </c>
       <c r="N21" s="5" t="inlineStr">
         <is>
@@ -4415,12 +4415,12 @@
       </c>
       <c r="U21" s="5" t="inlineStr">
         <is>
-          <t>Grupo Softbox</t>
+          <t>Grupo Mercurio York</t>
         </is>
       </c>
       <c r="V21" s="5" t="inlineStr">
         <is>
-          <t>Luizalabs</t>
+          <t>Agencia Mercurio York Viagens e Turismo Ltda</t>
         </is>
       </c>
       <c r="W21" s="5" t="inlineStr">
@@ -4430,11 +4430,11 @@
       </c>
       <c r="X21" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Azul Linhas Aereas</t>
         </is>
       </c>
       <c r="Y21" s="5" t="n">
-        <v>2250042719</v>
+        <v>733025258</v>
       </c>
       <c r="Z21" s="5" t="inlineStr">
         <is>
@@ -4447,16 +4447,16 @@
         </is>
       </c>
       <c r="AB21" s="5" t="n">
-        <v>1405.44</v>
+        <v>703.42</v>
       </c>
       <c r="AC21" s="5" t="n">
-        <v>74.59999999999999</v>
+        <v>46.36</v>
       </c>
       <c r="AD21" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE21" s="5" t="n">
-        <v>140.54</v>
+        <v>0</v>
       </c>
       <c r="AF21" s="5" t="n">
         <v>0</v>
@@ -4465,7 +4465,7 @@
         <v>0</v>
       </c>
       <c r="AH21" s="5" t="n">
-        <v>92.76000000000001</v>
+        <v>0</v>
       </c>
       <c r="AI21" s="5" t="inlineStr">
         <is>
@@ -4474,7 +4474,7 @@
       </c>
       <c r="AJ21" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 11/09/2025</t>
+          <t>Centro de custo não preenchido! (ACC01)</t>
         </is>
       </c>
       <c r="AK21" s="5" t="inlineStr">
@@ -4484,17 +4484,17 @@
       </c>
       <c r="AL21" s="5" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>Centro de custo</t>
         </is>
       </c>
       <c r="AM21" s="5" t="inlineStr">
         <is>
-          <t>Análise Benner</t>
+          <t>Falta de informação Gerencial</t>
         </is>
       </c>
       <c r="AN21" s="5" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Dados do Fornecedor</t>
         </is>
       </c>
       <c r="AO21" s="5" t="inlineStr">
@@ -4515,10 +4515,10 @@
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
-        <v>22910566</v>
+        <v>23079031</v>
       </c>
       <c r="B22" s="5" t="n">
-        <v>23683752</v>
+        <v>23830396</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
@@ -4526,10 +4526,10 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>45911.76108796296</v>
+        <v>45939.59543981482</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>45911.76306712963</v>
+        <v>45939.59658564815</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
@@ -4543,7 +4543,7 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>UJ2VYS</t>
+          <t>GHOQOV</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
@@ -4553,7 +4553,7 @@
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>Rodrigues Pinto/Cristian</t>
+          <t>ANGE ARAUJO/ENY</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -4567,7 +4567,7 @@
         </is>
       </c>
       <c r="M22" s="6" t="n">
-        <v>45911.25902777778</v>
+        <v>45939.08888888889</v>
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
@@ -4606,12 +4606,12 @@
       </c>
       <c r="U22" s="5" t="inlineStr">
         <is>
-          <t>Grupo Kontrip</t>
+          <t>Grupo Mercurio York</t>
         </is>
       </c>
       <c r="V22" s="5" t="inlineStr">
         <is>
-          <t>Kontrip - Vendas Cartao de Credito</t>
+          <t>Agencia Mercurio York Viagens e Turismo Ltda</t>
         </is>
       </c>
       <c r="W22" s="5" t="inlineStr">
@@ -4621,11 +4621,11 @@
       </c>
       <c r="X22" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Gol Linhas Aereas</t>
         </is>
       </c>
       <c r="Y22" s="5" t="n">
-        <v>852567250</v>
+        <v>2147038510</v>
       </c>
       <c r="Z22" s="5" t="inlineStr">
         <is>
@@ -4638,10 +4638,10 @@
         </is>
       </c>
       <c r="AB22" s="5" t="n">
-        <v>583</v>
+        <v>3759.86</v>
       </c>
       <c r="AC22" s="5" t="n">
-        <v>0</v>
+        <v>113.34</v>
       </c>
       <c r="AD22" s="5" t="n">
         <v>0</v>
@@ -4656,7 +4656,7 @@
         <v>0</v>
       </c>
       <c r="AH22" s="5" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="AI22" s="5" t="inlineStr">
         <is>
@@ -4665,7 +4665,7 @@
       </c>
       <c r="AJ22" s="5" t="inlineStr">
         <is>
-          <t>Pnr já existente. A duplicidade de rloc é permitida apenas 6 meses após o último pnr emitido</t>
+          <t>Centro de custo não preenchido! (ACC01)</t>
         </is>
       </c>
       <c r="AK22" s="5" t="inlineStr">
@@ -4675,17 +4675,17 @@
       </c>
       <c r="AL22" s="5" t="inlineStr">
         <is>
-          <t>Duplicidade de RLOC</t>
+          <t>Centro de custo</t>
         </is>
       </c>
       <c r="AM22" s="5" t="inlineStr">
         <is>
-          <t>Campo RLOC</t>
+          <t>Falta de informação Gerencial</t>
         </is>
       </c>
       <c r="AN22" s="5" t="inlineStr">
         <is>
-          <t>Duplicidade de Contabilização</t>
+          <t>Dados do Fornecedor</t>
         </is>
       </c>
       <c r="AO22" s="5" t="inlineStr">
@@ -4699,197 +4699,6 @@
         </is>
       </c>
       <c r="AQ22" s="5" t="inlineStr">
-        <is>
-          <t>Operações - KONTRIP</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="n">
-        <v>22909199</v>
-      </c>
-      <c r="B23" s="5" t="n">
-        <v>23682402</v>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>ACC01</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="n">
-        <v>45911.61663194445</v>
-      </c>
-      <c r="E23" s="6" t="n">
-        <v>45911.61732638889</v>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>0 a 02 dias</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>0 a 02 dias</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>PGLMHI</t>
-        </is>
-      </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>EBOOKING</t>
-        </is>
-      </c>
-      <c r="J23" s="5" t="inlineStr">
-        <is>
-          <t>FONTELES/WEYDSON</t>
-        </is>
-      </c>
-      <c r="K23" s="5" t="inlineStr">
-        <is>
-          <t>Kontrip</t>
-        </is>
-      </c>
-      <c r="L23" s="5" t="inlineStr">
-        <is>
-          <t>Kontrip</t>
-        </is>
-      </c>
-      <c r="M23" s="6" t="n">
-        <v>45911.53680555556</v>
-      </c>
-      <c r="N23" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O23" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P23" s="5" t="inlineStr">
-        <is>
-          <t>OFF LINE</t>
-        </is>
-      </c>
-      <c r="Q23" s="5" t="inlineStr">
-        <is>
-          <t>Cartão de crédito</t>
-        </is>
-      </c>
-      <c r="R23" s="5" t="inlineStr">
-        <is>
-          <t>Cartão de crédito</t>
-        </is>
-      </c>
-      <c r="S23" s="5" t="inlineStr">
-        <is>
-          <t>Aéreo</t>
-        </is>
-      </c>
-      <c r="T23" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="U23" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Kontrip</t>
-        </is>
-      </c>
-      <c r="V23" s="5" t="inlineStr">
-        <is>
-          <t>Instituto de Tecnologia Educacional</t>
-        </is>
-      </c>
-      <c r="W23" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X23" s="5" t="inlineStr">
-        <is>
-          <t>Azul Linhas Aereas</t>
-        </is>
-      </c>
-      <c r="Y23" s="5" t="n">
-        <v>863366431</v>
-      </c>
-      <c r="Z23" s="5" t="inlineStr">
-        <is>
-          <t>KONTRIP</t>
-        </is>
-      </c>
-      <c r="AA23" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB23" s="5" t="n">
-        <v>1421.17</v>
-      </c>
-      <c r="AC23" s="5" t="n">
-        <v>51.67</v>
-      </c>
-      <c r="AD23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH23" s="5" t="n">
-        <v>113.69</v>
-      </c>
-      <c r="AI23" s="5" t="inlineStr">
-        <is>
-          <t>obs</t>
-        </is>
-      </c>
-      <c r="AJ23" s="5" t="inlineStr">
-        <is>
-          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 11/09/2025</t>
-        </is>
-      </c>
-      <c r="AK23" s="5" t="inlineStr">
-        <is>
-          <t>KONTRIP</t>
-        </is>
-      </c>
-      <c r="AL23" s="5" t="inlineStr">
-        <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="AM23" s="5" t="inlineStr">
-        <is>
-          <t>Análise Benner</t>
-        </is>
-      </c>
-      <c r="AN23" s="5" t="inlineStr">
-        <is>
-          <t>Sistema</t>
-        </is>
-      </c>
-      <c r="AO23" s="5" t="inlineStr">
-        <is>
-          <t>Qualidade dos dados</t>
-        </is>
-      </c>
-      <c r="AP23" s="5" t="inlineStr">
-        <is>
-          <t>KONTRIP VIAGENS</t>
-        </is>
-      </c>
-      <c r="AQ23" s="5" t="inlineStr">
         <is>
           <t>Operações - KONTRIP</t>
         </is>

</xml_diff>

<commit_message>
Refresh Integration-Quality files, remove old scripts
Remove deprecated utility scripts and refresh Integration-Quality artifacts. Deleted legacy FCM control files and associated scripts, ecommerce data generator and POKEDEX population script. Updated Integration-Quality reporting code (4-envio_relatorios.py) to adjust recipient lists for several companies. Replaced/updated multiple binary report spreadsheets and dashboards, added new company report (Relatorio - INOVENTS.xlsx) and a set of PDF reports (Integration-Quality/PDFs) for May 4–18, 2026. These changes consolidate current reports and clean up unused tooling.
</commit_message>
<xml_diff>
--- a/Integration-Quality/EMPRESAS/Relatorio - KONTRIP VIAGENS.xlsx
+++ b/Integration-Quality/EMPRESAS/Relatorio - KONTRIP VIAGENS.xlsx
@@ -18,7 +18,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,9 +41,6 @@
     <font>
       <b val="1"/>
       <color rgb="00591F6A"/>
-    </font>
-    <font>
-      <color rgb="00FF0000"/>
     </font>
   </fonts>
   <fills count="4">
@@ -93,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -109,9 +106,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -479,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ21"/>
+  <dimension ref="A1:AQ20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -701,10 +695,10 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
-        <v>24507872</v>
+        <v>24599778</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>25322150</v>
+        <v>25425830</v>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
@@ -712,24 +706,24 @@
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>46139.80263888889</v>
+        <v>46157.62378472222</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>46139.80475694445</v>
+        <v>46157.62619212963</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>MYHCPS</t>
+          <t>YYTUDZ</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -739,7 +733,7 @@
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>MOREIRA DA SILVA/EDUARDO</t>
+          <t>CONCEIÇÃO DOS SANTOS/JOEL</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -753,7 +747,7 @@
         </is>
       </c>
       <c r="M2" s="6" t="n">
-        <v>46139.30208333334</v>
+        <v>46157.12222222222</v>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
@@ -792,12 +786,12 @@
       </c>
       <c r="U2" s="5" t="inlineStr">
         <is>
-          <t>Grupo Kontrip</t>
+          <t>Grupo Sacs</t>
         </is>
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>M3. Business Group Ltda</t>
+          <t>Sacs Construcao e Montagem Ltda</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -807,11 +801,11 @@
       </c>
       <c r="X2" s="5" t="inlineStr">
         <is>
-          <t>Gol Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y2" s="5" t="n">
-        <v>2302657077</v>
+        <v>2286891563</v>
       </c>
       <c r="Z2" s="5" t="inlineStr">
         <is>
@@ -824,10 +818,10 @@
         </is>
       </c>
       <c r="AB2" s="5" t="n">
-        <v>3548.07</v>
+        <v>1134.96</v>
       </c>
       <c r="AC2" s="5" t="n">
-        <v>88.2</v>
+        <v>86.36</v>
       </c>
       <c r="AD2" s="5" t="n">
         <v>0</v>
@@ -842,7 +836,7 @@
         <v>0</v>
       </c>
       <c r="AH2" s="5" t="n">
-        <v>324.35</v>
+        <v>111.76</v>
       </c>
       <c r="AI2" s="5" t="inlineStr">
         <is>
@@ -851,7 +845,7 @@
       </c>
       <c r="AJ2" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 27/04/2026</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 15/05/2026</t>
         </is>
       </c>
       <c r="AK2" s="5" t="inlineStr">
@@ -892,10 +886,10 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>24494682</v>
+        <v>24598779</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>25306200</v>
+        <v>25424773</v>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
@@ -903,10 +897,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>46136.61430555556</v>
+        <v>46157.48453703704</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>46137.081875</v>
+        <v>46157.48613425926</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
@@ -920,34 +914,36 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>EREAEB</t>
+          <t>WEGNJR</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>WOOBA</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>AGUIAR LINDENBERG/CARLOS MR</t>
+          <t>HENRIK PROENÇA FERNA/IGOR</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>Toou</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>Toou</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="M3" s="6" t="n">
-        <v>46136.60927083333</v>
-      </c>
-      <c r="N3" s="5" t="n">
-        <v>1670</v>
+        <v>46157.48333333333</v>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
@@ -966,7 +962,7 @@
       </c>
       <c r="R3" s="5" t="inlineStr">
         <is>
-          <t>Cartão AMEX</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="S3" s="5" t="inlineStr">
@@ -981,12 +977,12 @@
       </c>
       <c r="U3" s="5" t="inlineStr">
         <is>
-          <t>Grupo Rede Gazeta</t>
+          <t>Grupo Kontrip</t>
         </is>
       </c>
       <c r="V3" s="5" t="inlineStr">
         <is>
-          <t>Tv Gazeta</t>
+          <t>Innova Educacao Comercio De Produtos Educacionais Ltda</t>
         </is>
       </c>
       <c r="W3" s="5" t="inlineStr">
@@ -996,11 +992,11 @@
       </c>
       <c r="X3" s="5" t="inlineStr">
         <is>
-          <t>Gol Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y3" s="5" t="n">
-        <v>2302468462</v>
+        <v>2286874083</v>
       </c>
       <c r="Z3" s="5" t="inlineStr">
         <is>
@@ -1013,10 +1009,10 @@
         </is>
       </c>
       <c r="AB3" s="5" t="n">
-        <v>283.4</v>
+        <v>1469.9</v>
       </c>
       <c r="AC3" s="5" t="n">
-        <v>62.14</v>
+        <v>450</v>
       </c>
       <c r="AD3" s="5" t="n">
         <v>0</v>
@@ -1031,16 +1027,16 @@
         <v>0</v>
       </c>
       <c r="AH3" s="5" t="n">
-        <v>25.51</v>
+        <v>40</v>
       </c>
       <c r="AI3" s="5" t="inlineStr">
         <is>
-          <t>Reserva importada do Sistema WOOBA. Id: 4598</t>
+          <t>obs</t>
         </is>
       </c>
       <c r="AJ3" s="5" t="inlineStr">
         <is>
-          <t>Empenho/departamento não preenchido! (ACC02) Matrícula não preenchida! (ACC02)</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 15/05/2026</t>
         </is>
       </c>
       <c r="AK3" s="5" t="inlineStr">
@@ -1050,17 +1046,17 @@
       </c>
       <c r="AL3" s="5" t="inlineStr">
         <is>
-          <t>Mais de um campo não preenchido</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM3" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN3" s="5" t="inlineStr">
         <is>
-          <t>Dados do Fornecedor</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO3" s="5" t="inlineStr">
@@ -1081,21 +1077,21 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>24494682</v>
+        <v>24544417</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>25306201</v>
+        <v>25367756</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>ACC02</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>46136.61430555556</v>
+        <v>46148.63471064815</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>46137.081875</v>
+        <v>46157.41923611111</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
@@ -1104,39 +1100,41 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>EREAEB</t>
+          <t>AJJ47Z01</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>WOOBA</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>AGUIAR LINDENBERG/CAROLINA MRS</t>
+          <t>TEIXEIRA DA SILVA/NILTON</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>Toou</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>Toou</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="M4" s="6" t="n">
-        <v>46136.60927083333</v>
-      </c>
-      <c r="N4" s="5" t="n">
-        <v>1670</v>
+        <v>46148.13402777778</v>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1153,7 @@
       </c>
       <c r="R4" s="5" t="inlineStr">
         <is>
-          <t>Cartão AMEX</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="S4" s="5" t="inlineStr">
@@ -1165,17 +1163,17 @@
       </c>
       <c r="T4" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>Grupo Rede Gazeta</t>
+          <t>Grupo Kontrip</t>
         </is>
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>Tv Gazeta</t>
+          <t>Kontrip - Vendas Cartao de Credito</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1185,11 +1183,11 @@
       </c>
       <c r="X4" s="5" t="inlineStr">
         <is>
-          <t>Gol Linhas Aereas</t>
+          <t>Azul Linhas Aereas</t>
         </is>
       </c>
       <c r="Y4" s="5" t="n">
-        <v>2302468463</v>
+        <v>389040422</v>
       </c>
       <c r="Z4" s="5" t="inlineStr">
         <is>
@@ -1202,10 +1200,10 @@
         </is>
       </c>
       <c r="AB4" s="5" t="n">
-        <v>283.4</v>
+        <v>119.88</v>
       </c>
       <c r="AC4" s="5" t="n">
-        <v>62.14</v>
+        <v>122.52</v>
       </c>
       <c r="AD4" s="5" t="n">
         <v>0</v>
@@ -1220,16 +1218,16 @@
         <v>0</v>
       </c>
       <c r="AH4" s="5" t="n">
-        <v>25.51</v>
+        <v>11.99</v>
       </c>
       <c r="AI4" s="5" t="inlineStr">
         <is>
-          <t>Reserva importada do Sistema WOOBA. Id: 4598</t>
+          <t>obs</t>
         </is>
       </c>
       <c r="AJ4" s="5" t="inlineStr">
         <is>
-          <t>Empenho/departamento não preenchido! (ACC02) Matrícula não preenchida! (ACC02)</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 06/05/2026</t>
         </is>
       </c>
       <c r="AK4" s="5" t="inlineStr">
@@ -1239,17 +1237,17 @@
       </c>
       <c r="AL4" s="5" t="inlineStr">
         <is>
-          <t>Mais de um campo não preenchido</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM4" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN4" s="5" t="inlineStr">
         <is>
-          <t>Dados do Fornecedor</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO4" s="5" t="inlineStr">
@@ -1270,10 +1268,10 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>24405792</v>
+        <v>24605123</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>25206427</v>
+        <v>25431958</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
@@ -1281,48 +1279,48 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>46118.43357638889</v>
+        <v>46158.55533564815</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>46126.354375</v>
+        <v>46158.55716435185</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>16 a 23 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>LPHLSM</t>
+          <t>CQC3WX</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>ONEIDE FRANCISCO BASSO</t>
+          <t>LIMA ROCHA/GERSON</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="M5" s="6" t="n">
-        <v>46114.43333333333</v>
+        <v>46158.05347222222</v>
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
@@ -1361,12 +1359,12 @@
       </c>
       <c r="U5" s="5" t="inlineStr">
         <is>
-          <t>Grupo Zupper</t>
+          <t>Grupo Kontrip</t>
         </is>
       </c>
       <c r="V5" s="5" t="inlineStr">
         <is>
-          <t>Basso e Pancotte</t>
+          <t>Red Engenharia Industrial Especializada Ltda</t>
         </is>
       </c>
       <c r="W5" s="5" t="inlineStr">
@@ -1376,11 +1374,11 @@
       </c>
       <c r="X5" s="5" t="inlineStr">
         <is>
-          <t>Gol Linhas Aereas</t>
+          <t>Azul Linhas Aereas</t>
         </is>
       </c>
       <c r="Y5" s="5" t="n">
-        <v>2301086081</v>
+        <v>464342178</v>
       </c>
       <c r="Z5" s="5" t="inlineStr">
         <is>
@@ -1393,10 +1391,10 @@
         </is>
       </c>
       <c r="AB5" s="5" t="n">
-        <v>2724.34</v>
+        <v>2089.35</v>
       </c>
       <c r="AC5" s="5" t="n">
-        <v>93</v>
+        <v>0</v>
       </c>
       <c r="AD5" s="5" t="n">
         <v>0</v>
@@ -1411,16 +1409,16 @@
         <v>0</v>
       </c>
       <c r="AH5" s="5" t="n">
-        <v>245.19</v>
+        <v>40</v>
       </c>
       <c r="AI5" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>obs</t>
         </is>
       </c>
       <c r="AJ5" s="5" t="inlineStr">
         <is>
-          <t>Could not convert variant of type (Null) into type (OleStr)</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 16/05/2026</t>
         </is>
       </c>
       <c r="AK5" s="5" t="inlineStr">
@@ -1461,10 +1459,10 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>24494683</v>
+        <v>24605228</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>25306202</v>
+        <v>25432067</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
@@ -1472,51 +1470,53 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>46136.6143287037</v>
+        <v>46158.56228009259</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>46137.08188657407</v>
+        <v>46158.56333333333</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>IVQEVB</t>
+          <t>IGDZGY</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>WOOBA</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>AGUIAR LINDENBERG/CARLOS MR</t>
+          <t>FERNANDES/PATRICK</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>Toou</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>Toou</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="M6" s="6" t="n">
-        <v>46136.61043981482</v>
-      </c>
-      <c r="N6" s="5" t="n">
-        <v>1671</v>
+        <v>46158.06111111111</v>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="R6" s="5" t="inlineStr">
         <is>
-          <t>Cartão AMEX</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="S6" s="5" t="inlineStr">
@@ -1550,12 +1550,12 @@
       </c>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>Grupo Rede Gazeta</t>
+          <t>Grupo Kontrip</t>
         </is>
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>Tv Gazeta</t>
+          <t>Red Engenharia Industrial Especializada Ltda</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1565,11 +1565,11 @@
       </c>
       <c r="X6" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Azul Linhas Aereas</t>
         </is>
       </c>
       <c r="Y6" s="5" t="n">
-        <v>2283969580</v>
+        <v>731623659</v>
       </c>
       <c r="Z6" s="5" t="inlineStr">
         <is>
@@ -1582,10 +1582,10 @@
         </is>
       </c>
       <c r="AB6" s="5" t="n">
-        <v>675.5599999999999</v>
+        <v>2100.54</v>
       </c>
       <c r="AC6" s="5" t="n">
-        <v>54.09</v>
+        <v>450</v>
       </c>
       <c r="AD6" s="5" t="n">
         <v>0</v>
@@ -1600,16 +1600,16 @@
         <v>0</v>
       </c>
       <c r="AH6" s="5" t="n">
-        <v>74.31</v>
+        <v>40</v>
       </c>
       <c r="AI6" s="5" t="inlineStr">
         <is>
-          <t>Reserva importada do Sistema WOOBA. Id: 4600</t>
+          <t>obs</t>
         </is>
       </c>
       <c r="AJ6" s="5" t="inlineStr">
         <is>
-          <t>Empenho/departamento não preenchido! (ACC02) Matrícula não preenchida! (ACC02)</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 16/05/2026</t>
         </is>
       </c>
       <c r="AK6" s="5" t="inlineStr">
@@ -1619,17 +1619,17 @@
       </c>
       <c r="AL6" s="5" t="inlineStr">
         <is>
-          <t>Mais de um campo não preenchido</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM6" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN6" s="5" t="inlineStr">
         <is>
-          <t>Dados do Fornecedor</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO6" s="5" t="inlineStr">
@@ -1650,62 +1650,64 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>24494683</v>
+        <v>24605018</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>25306203</v>
+        <v>25431828</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>ACC02</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>46136.6143287037</v>
+        <v>46158.53730324074</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>46137.08188657407</v>
+        <v>46158.53851851852</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>IVQEVB</t>
+          <t>MNBXNW</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>WOOBA</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>AGUIAR LINDENBERG/CAROLINA MRS</t>
+          <t>Teotonio Junior/Epaminondas</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>Toou</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>Toou</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="M7" s="6" t="n">
-        <v>46136.61043981482</v>
-      </c>
-      <c r="N7" s="5" t="n">
-        <v>1671</v>
+        <v>46158.53611111111</v>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
@@ -1724,7 +1726,7 @@
       </c>
       <c r="R7" s="5" t="inlineStr">
         <is>
-          <t>Cartão AMEX</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="S7" s="5" t="inlineStr">
@@ -1739,12 +1741,12 @@
       </c>
       <c r="U7" s="5" t="inlineStr">
         <is>
-          <t>Grupo Rede Gazeta</t>
+          <t>Grupo Kontrip</t>
         </is>
       </c>
       <c r="V7" s="5" t="inlineStr">
         <is>
-          <t>Tv Gazeta</t>
+          <t>Kontrip - Vendas Cartao de Credito</t>
         </is>
       </c>
       <c r="W7" s="5" t="inlineStr">
@@ -1754,11 +1756,11 @@
       </c>
       <c r="X7" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Gol Linhas Aereas</t>
         </is>
       </c>
       <c r="Y7" s="5" t="n">
-        <v>2283969581</v>
+        <v>2303902227</v>
       </c>
       <c r="Z7" s="5" t="inlineStr">
         <is>
@@ -1771,10 +1773,10 @@
         </is>
       </c>
       <c r="AB7" s="5" t="n">
-        <v>675.5599999999999</v>
+        <v>2155.06</v>
       </c>
       <c r="AC7" s="5" t="n">
-        <v>54.09</v>
+        <v>33.64</v>
       </c>
       <c r="AD7" s="5" t="n">
         <v>0</v>
@@ -1789,16 +1791,16 @@
         <v>0</v>
       </c>
       <c r="AH7" s="5" t="n">
-        <v>74.31</v>
+        <v>387.92</v>
       </c>
       <c r="AI7" s="5" t="inlineStr">
         <is>
-          <t>Reserva importada do Sistema WOOBA. Id: 4600</t>
+          <t>obs</t>
         </is>
       </c>
       <c r="AJ7" s="5" t="inlineStr">
         <is>
-          <t>Empenho/departamento não preenchido! (ACC02) Matrícula não preenchida! (ACC02)</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 16/05/2026</t>
         </is>
       </c>
       <c r="AK7" s="5" t="inlineStr">
@@ -1808,17 +1810,17 @@
       </c>
       <c r="AL7" s="5" t="inlineStr">
         <is>
-          <t>Mais de um campo não preenchido</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM7" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN7" s="5" t="inlineStr">
         <is>
-          <t>Dados do Fornecedor</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO7" s="5" t="inlineStr">
@@ -1839,21 +1841,21 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
-        <v>24507657</v>
+        <v>24605018</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>25321844</v>
+        <v>25431829</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>ACC01</t>
+          <t>ACC02</t>
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>46139.76956018519</v>
+        <v>46158.53730324074</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>46139.77182870371</v>
+        <v>46158.53851851852</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
@@ -1867,7 +1869,7 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>LA9576012ODBA</t>
+          <t>MNBXNW</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -1877,7 +1879,7 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Abdallah Mourad/Himad</t>
+          <t>Augusto Rocha e Silva/Filipe</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1891,7 +1893,7 @@
         </is>
       </c>
       <c r="M8" s="6" t="n">
-        <v>46139.11805555555</v>
+        <v>46158.53611111111</v>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
@@ -1935,7 +1937,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>Cda</t>
+          <t>Kontrip - Vendas Cartao de Credito</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1945,11 +1947,11 @@
       </c>
       <c r="X8" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Gol Linhas Aereas</t>
         </is>
       </c>
       <c r="Y8" s="5" t="n">
-        <v>2284367251</v>
+        <v>2303902228</v>
       </c>
       <c r="Z8" s="5" t="inlineStr">
         <is>
@@ -1962,16 +1964,16 @@
         </is>
       </c>
       <c r="AB8" s="5" t="n">
-        <v>724.88</v>
+        <v>2155.06</v>
       </c>
       <c r="AC8" s="5" t="n">
-        <v>112.56</v>
+        <v>33.64</v>
       </c>
       <c r="AD8" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE8" s="5" t="n">
-        <v>72.48</v>
+        <v>0</v>
       </c>
       <c r="AF8" s="5" t="n">
         <v>0</v>
@@ -1980,7 +1982,7 @@
         <v>0</v>
       </c>
       <c r="AH8" s="5" t="n">
-        <v>51.83</v>
+        <v>0</v>
       </c>
       <c r="AI8" s="5" t="inlineStr">
         <is>
@@ -1989,7 +1991,7 @@
       </c>
       <c r="AJ8" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 27/04/2026</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 16/05/2026</t>
         </is>
       </c>
       <c r="AK8" s="5" t="inlineStr">
@@ -2030,21 +2032,21 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>24494720</v>
+        <v>24601662</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>25306270</v>
+        <v>25428031</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>46136.61736111111</v>
+        <v>46157.81648148148</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>46136.62313657408</v>
+        <v>46157.81768518518</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
@@ -2058,31 +2060,31 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>6EWFOD</t>
+          <t>CGL5YI</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>VANESSA CHAVES</t>
+          <t>MARIA DUARTE ALVES/JESSICA</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="M9" s="6" t="n">
-        <v>46135.61736111111</v>
+        <v>46157.31458333333</v>
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
@@ -2126,7 +2128,7 @@
       </c>
       <c r="V9" s="5" t="inlineStr">
         <is>
-          <t>Kontrip - Vendas Cartao de Credito</t>
+          <t>Lpe Engenharia e Consultoria Ltda</t>
         </is>
       </c>
       <c r="W9" s="5" t="inlineStr">
@@ -2136,11 +2138,11 @@
       </c>
       <c r="X9" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Azul Linhas Aereas</t>
         </is>
       </c>
       <c r="Y9" s="5" t="n">
-        <v>2283882921</v>
+        <v>137324207</v>
       </c>
       <c r="Z9" s="5" t="inlineStr">
         <is>
@@ -2153,16 +2155,16 @@
         </is>
       </c>
       <c r="AB9" s="5" t="n">
-        <v>993.24</v>
+        <v>507.15</v>
       </c>
       <c r="AC9" s="5" t="n">
-        <v>60.54</v>
+        <v>48.63</v>
       </c>
       <c r="AD9" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE9" s="5" t="n">
-        <v>99.31999999999999</v>
+        <v>0</v>
       </c>
       <c r="AF9" s="5" t="n">
         <v>0</v>
@@ -2171,16 +2173,16 @@
         <v>0</v>
       </c>
       <c r="AH9" s="5" t="n">
-        <v>71.02</v>
+        <v>32.14</v>
       </c>
       <c r="AI9" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>obs</t>
         </is>
       </c>
       <c r="AJ9" s="5" t="inlineStr">
         <is>
-          <t>36Faltou informar rateio de centro de custo/projeto abaixo da accounting</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 15/05/2026</t>
         </is>
       </c>
       <c r="AK9" s="5" t="inlineStr">
@@ -2190,17 +2192,17 @@
       </c>
       <c r="AL9" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM9" s="5" t="inlineStr">
         <is>
-          <t>Rateio de centro de custo/projeto</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN9" s="5" t="inlineStr">
         <is>
-          <t>Dados Gerenciais</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO9" s="5" t="inlineStr">
@@ -2221,21 +2223,21 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>24493854</v>
+        <v>24601071</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>25305308</v>
+        <v>25427420</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>46136.50267361111</v>
+        <v>46157.79983796296</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>46136.50651620371</v>
+        <v>46157.80114583333</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
@@ -2249,31 +2251,31 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>AJM35Z</t>
+          <t>FAJPZW</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>PAULO HENRIQUE FERREIRA VAZZOLER</t>
+          <t>MARIA DUARTE ALVES/JESSICA</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="M10" s="6" t="n">
-        <v>46133.50208333333</v>
+        <v>46157.29861111111</v>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
@@ -2317,7 +2319,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>Kontrip - Vendas Cartao de Credito</t>
+          <t>Lpe Engenharia e Consultoria Ltda</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -2327,11 +2329,11 @@
       </c>
       <c r="X10" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y10" s="5" t="n">
-        <v>3025305307</v>
+        <v>228688497</v>
       </c>
       <c r="Z10" s="5" t="inlineStr">
         <is>
@@ -2344,10 +2346,10 @@
         </is>
       </c>
       <c r="AB10" s="5" t="n">
-        <v>412.12</v>
+        <v>559.17</v>
       </c>
       <c r="AC10" s="5" t="n">
-        <v>48.75</v>
+        <v>62.14</v>
       </c>
       <c r="AD10" s="5" t="n">
         <v>0</v>
@@ -2362,16 +2364,16 @@
         <v>0</v>
       </c>
       <c r="AH10" s="5" t="n">
-        <v>41.21</v>
+        <v>42.22</v>
       </c>
       <c r="AI10" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>obs</t>
         </is>
       </c>
       <c r="AJ10" s="5" t="inlineStr">
         <is>
-          <t>36Faltou informar rateio de centro de custo/projeto abaixo da accounting</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 15/05/2026</t>
         </is>
       </c>
       <c r="AK10" s="5" t="inlineStr">
@@ -2381,17 +2383,17 @@
       </c>
       <c r="AL10" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM10" s="5" t="inlineStr">
         <is>
-          <t>Rateio de centro de custo/projeto</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN10" s="5" t="inlineStr">
         <is>
-          <t>Dados Gerenciais</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO10" s="5" t="inlineStr">
@@ -2412,10 +2414,10 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
-        <v>24419465</v>
+        <v>24601282</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>25221482</v>
+        <v>25427630</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
@@ -2423,24 +2425,24 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>46120.66405092592</v>
+        <v>46157.80396990741</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>46123.73384259259</v>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>16 a 23 dias</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>16 a 23 dias</t>
+        <v>46157.80489583333</v>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>03 a 05 dias</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>MMTY6D01</t>
+          <t>OG284Y</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
@@ -2450,7 +2452,7 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>SANTOS DE OLIVEIRA PITANGA/CAIQUE</t>
+          <t>MARIA DUARTE ALVES/JESSICA</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
@@ -2464,7 +2466,7 @@
         </is>
       </c>
       <c r="M11" s="6" t="n">
-        <v>46120.1625</v>
+        <v>46157.30347222222</v>
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
@@ -2498,7 +2500,7 @@
       </c>
       <c r="T11" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U11" s="5" t="inlineStr">
@@ -2508,7 +2510,7 @@
       </c>
       <c r="V11" s="5" t="inlineStr">
         <is>
-          <t>Wps Brasil Ltda</t>
+          <t>Lpe Engenharia e Consultoria Ltda</t>
         </is>
       </c>
       <c r="W11" s="5" t="inlineStr">
@@ -2522,7 +2524,7 @@
         </is>
       </c>
       <c r="Y11" s="5" t="n">
-        <v>495316528</v>
+        <v>538633897</v>
       </c>
       <c r="Z11" s="5" t="inlineStr">
         <is>
@@ -2535,10 +2537,10 @@
         </is>
       </c>
       <c r="AB11" s="5" t="n">
-        <v>1202.79</v>
+        <v>586.16</v>
       </c>
       <c r="AC11" s="5" t="n">
-        <v>113.26</v>
+        <v>48.63</v>
       </c>
       <c r="AD11" s="5" t="n">
         <v>0</v>
@@ -2553,7 +2555,7 @@
         <v>0</v>
       </c>
       <c r="AH11" s="5" t="n">
-        <v>108.25</v>
+        <v>39.25</v>
       </c>
       <c r="AI11" s="5" t="inlineStr">
         <is>
@@ -2562,7 +2564,7 @@
       </c>
       <c r="AJ11" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 08/04/2026</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 15/05/2026</t>
         </is>
       </c>
       <c r="AK11" s="5" t="inlineStr">
@@ -2603,10 +2605,10 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
-        <v>24493797</v>
+        <v>24601487</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>25305242</v>
+        <v>25427840</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
@@ -2614,10 +2616,10 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>46136.49399305556</v>
+        <v>46157.80961805556</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>46136.49840277778</v>
+        <v>46157.81137731481</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
@@ -2631,31 +2633,31 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> WJK7MS</t>
+          <t>FDNIBJ</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>VIVIAN LUTGARD ZACCONI AQUINO</t>
+          <t>MARIA DUARTE ALVES/JESSICA</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="M12" s="6" t="n">
-        <v>46132.49375</v>
+        <v>46157.30833333333</v>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
@@ -2699,7 +2701,7 @@
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>E-rural Atividades de Internet</t>
+          <t>Lpe Engenharia e Consultoria Ltda</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -2709,11 +2711,11 @@
       </c>
       <c r="X12" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y12" s="5" t="n">
-        <v>3025305241</v>
+        <v>228688516</v>
       </c>
       <c r="Z12" s="5" t="inlineStr">
         <is>
@@ -2726,10 +2728,10 @@
         </is>
       </c>
       <c r="AB12" s="5" t="n">
-        <v>410</v>
+        <v>462.28</v>
       </c>
       <c r="AC12" s="5" t="n">
-        <v>32.87</v>
+        <v>62.14</v>
       </c>
       <c r="AD12" s="5" t="n">
         <v>0</v>
@@ -2744,16 +2746,16 @@
         <v>0</v>
       </c>
       <c r="AH12" s="5" t="n">
-        <v>82</v>
+        <v>34.35</v>
       </c>
       <c r="AI12" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>obs</t>
         </is>
       </c>
       <c r="AJ12" s="5" t="inlineStr">
         <is>
-          <t>36Faltou informar rateio de centro de custo/projeto abaixo da accounting</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 15/05/2026</t>
         </is>
       </c>
       <c r="AK12" s="5" t="inlineStr">
@@ -2763,17 +2765,17 @@
       </c>
       <c r="AL12" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM12" s="5" t="inlineStr">
         <is>
-          <t>Rateio de centro de custo/projeto</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN12" s="5" t="inlineStr">
         <is>
-          <t>Dados Gerenciais</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO12" s="5" t="inlineStr">
@@ -2794,21 +2796,21 @@
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
-        <v>24493797</v>
+        <v>24598641</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>25305244</v>
+        <v>25424592</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>ACC02</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>46136.49399305556</v>
+        <v>46157.45399305555</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>46136.49840277778</v>
+        <v>46157.45474537037</v>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
@@ -2822,31 +2824,31 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> WJK7MS</t>
+          <t>JZVCLK</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>MATHEUS SEROA</t>
+          <t>Henrique Peres dos Santos/Iago</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="M13" s="6" t="n">
-        <v>46132.49375</v>
+        <v>46157.45208333333</v>
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
@@ -2890,7 +2892,7 @@
       </c>
       <c r="V13" s="5" t="inlineStr">
         <is>
-          <t>E-rural Atividades de Internet</t>
+          <t>Lobov Cientifica</t>
         </is>
       </c>
       <c r="W13" s="5" t="inlineStr">
@@ -2900,11 +2902,11 @@
       </c>
       <c r="X13" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y13" s="5" t="n">
-        <v>3025305241</v>
+        <v>2286866372</v>
       </c>
       <c r="Z13" s="5" t="inlineStr">
         <is>
@@ -2917,10 +2919,10 @@
         </is>
       </c>
       <c r="AB13" s="5" t="n">
-        <v>410</v>
+        <v>1020.89</v>
       </c>
       <c r="AC13" s="5" t="n">
-        <v>32.87</v>
+        <v>500</v>
       </c>
       <c r="AD13" s="5" t="n">
         <v>0</v>
@@ -2935,16 +2937,16 @@
         <v>0</v>
       </c>
       <c r="AH13" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="AI13" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>obs</t>
         </is>
       </c>
       <c r="AJ13" s="5" t="inlineStr">
         <is>
-          <t>36Faltou informar rateio de centro de custo/projeto abaixo da accounting</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 15/05/2026</t>
         </is>
       </c>
       <c r="AK13" s="5" t="inlineStr">
@@ -2954,17 +2956,17 @@
       </c>
       <c r="AL13" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM13" s="5" t="inlineStr">
         <is>
-          <t>Rateio de centro de custo/projeto</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN13" s="5" t="inlineStr">
         <is>
-          <t>Dados Gerenciais</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO13" s="5" t="inlineStr">
@@ -2985,21 +2987,21 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
-        <v>24494430</v>
+        <v>24578818</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>25305913</v>
+        <v>25402494</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>46136.5408912037</v>
+        <v>46154.61798611111</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>46136.54615740741</v>
+        <v>46155.53385416666</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
@@ -3008,36 +3010,36 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>AGFPPI</t>
+          <t>ETMIMA02</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>JOSE LUIZ DE MOURA FALEIROS JUNIOR</t>
+          <t>Zampirollo Neto/Octavio</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Juliana Cardoso</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Juliana Cardoso</t>
         </is>
       </c>
       <c r="M14" s="6" t="n">
-        <v>46135.54027777778</v>
+        <v>46149.11736111111</v>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
@@ -3081,7 +3083,7 @@
       </c>
       <c r="V14" s="5" t="inlineStr">
         <is>
-          <t>Faculdade Baiana de Direito</t>
+          <t>Grant Thornton Auditores Independentes</t>
         </is>
       </c>
       <c r="W14" s="5" t="inlineStr">
@@ -3091,11 +3093,11 @@
       </c>
       <c r="X14" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y14" s="5" t="n">
-        <v>3025305912</v>
+        <v>2286408382</v>
       </c>
       <c r="Z14" s="5" t="inlineStr">
         <is>
@@ -3108,10 +3110,10 @@
         </is>
       </c>
       <c r="AB14" s="5" t="n">
-        <v>1082.34</v>
+        <v>838.88</v>
       </c>
       <c r="AC14" s="5" t="n">
-        <v>86.28</v>
+        <v>450</v>
       </c>
       <c r="AD14" s="5" t="n">
         <v>0</v>
@@ -3126,16 +3128,16 @@
         <v>0</v>
       </c>
       <c r="AH14" s="5" t="n">
-        <v>108.23</v>
+        <v>40</v>
       </c>
       <c r="AI14" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>obs</t>
         </is>
       </c>
       <c r="AJ14" s="5" t="inlineStr">
         <is>
-          <t>36Faltou informar rateio de centro de custo/projeto abaixo da accounting</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 07/05/2026</t>
         </is>
       </c>
       <c r="AK14" s="5" t="inlineStr">
@@ -3145,17 +3147,17 @@
       </c>
       <c r="AL14" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="AM14" s="5" t="inlineStr">
         <is>
-          <t>Rateio de centro de custo/projeto</t>
+          <t>Análise Benner</t>
         </is>
       </c>
       <c r="AN14" s="5" t="inlineStr">
         <is>
-          <t>Dados Gerenciais</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO14" s="5" t="inlineStr">
@@ -3176,21 +3178,21 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
-        <v>24494198</v>
+        <v>24600478</v>
       </c>
       <c r="B15" s="5" t="n">
-        <v>25305685</v>
+        <v>25426738</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>46136.52075231481</v>
+        <v>46157.72592592592</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>46136.52525462963</v>
+        <v>46157.729375</v>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
@@ -3204,7 +3206,7 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>IMC7VW</t>
+          <t>LA9573774CAIL</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -3214,21 +3216,21 @@
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>ANDERSON BEZERRA DE OLIVEIRA</t>
+          <t>MIGUEL DE DEUS</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Juliana Cardoso</t>
         </is>
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Juliana Cardoso</t>
         </is>
       </c>
       <c r="M15" s="6" t="n">
-        <v>46135.52013888889</v>
+        <v>46156.72569444445</v>
       </c>
       <c r="N15" s="5" t="inlineStr">
         <is>
@@ -3272,7 +3274,7 @@
       </c>
       <c r="V15" s="5" t="inlineStr">
         <is>
-          <t>Red Engenharia Industrial Especializada Ltda</t>
+          <t>2ms - Engenharia</t>
         </is>
       </c>
       <c r="W15" s="5" t="inlineStr">
@@ -3282,11 +3284,11 @@
       </c>
       <c r="X15" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y15" s="5" t="n">
-        <v>3025305683</v>
+        <v>2286703454</v>
       </c>
       <c r="Z15" s="5" t="inlineStr">
         <is>
@@ -3299,16 +3301,16 @@
         </is>
       </c>
       <c r="AB15" s="5" t="n">
-        <v>3893.62</v>
+        <v>515.96</v>
       </c>
       <c r="AC15" s="5" t="n">
-        <v>107.89</v>
+        <v>62.14</v>
       </c>
       <c r="AD15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE15" s="5" t="n">
-        <v>0</v>
+        <v>51.59</v>
       </c>
       <c r="AF15" s="5" t="n">
         <v>0</v>
@@ -3317,7 +3319,7 @@
         <v>0</v>
       </c>
       <c r="AH15" s="5" t="n">
-        <v>389.36</v>
+        <v>73.78</v>
       </c>
       <c r="AI15" s="5" t="inlineStr">
         <is>
@@ -3367,21 +3369,21 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
-        <v>24493870</v>
+        <v>24600478</v>
       </c>
       <c r="B16" s="5" t="n">
-        <v>25305316</v>
+        <v>25426741</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>ACC02</t>
         </is>
       </c>
       <c r="D16" s="6" t="n">
-        <v>46136.50516203704</v>
+        <v>46157.72592592592</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>46136.50883101852</v>
+        <v>46157.729375</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -3395,7 +3397,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>BQRKTH</t>
+          <t>LA9573774CAIL</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
@@ -3405,21 +3407,21 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>MIZAEL LIMA DOS REIS</t>
+          <t>SILVIA SANTOS</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Juliana Cardoso</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Juliana Cardoso</t>
         </is>
       </c>
       <c r="M16" s="6" t="n">
-        <v>46134.50486111111</v>
+        <v>46156.72569444445</v>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
@@ -3463,7 +3465,7 @@
       </c>
       <c r="V16" s="5" t="inlineStr">
         <is>
-          <t>Marques e Bezerra Ltda</t>
+          <t>2ms - Engenharia</t>
         </is>
       </c>
       <c r="W16" s="5" t="inlineStr">
@@ -3473,11 +3475,11 @@
       </c>
       <c r="X16" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y16" s="5" t="n">
-        <v>3025305315</v>
+        <v>2286703455</v>
       </c>
       <c r="Z16" s="5" t="inlineStr">
         <is>
@@ -3490,16 +3492,16 @@
         </is>
       </c>
       <c r="AB16" s="5" t="n">
-        <v>1873.62</v>
+        <v>515.96</v>
       </c>
       <c r="AC16" s="5" t="n">
-        <v>55.17</v>
+        <v>62.14</v>
       </c>
       <c r="AD16" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE16" s="5" t="n">
-        <v>0</v>
+        <v>51.59</v>
       </c>
       <c r="AF16" s="5" t="n">
         <v>0</v>
@@ -3508,7 +3510,7 @@
         <v>0</v>
       </c>
       <c r="AH16" s="5" t="n">
-        <v>187.36</v>
+        <v>0</v>
       </c>
       <c r="AI16" s="5" t="inlineStr">
         <is>
@@ -3558,10 +3560,10 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
-        <v>24493523</v>
+        <v>24599775</v>
       </c>
       <c r="B17" s="5" t="n">
-        <v>25304914</v>
+        <v>25425828</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
@@ -3569,10 +3571,10 @@
         </is>
       </c>
       <c r="D17" s="6" t="n">
-        <v>46136.43653935185</v>
+        <v>46157.62344907408</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>46136.44121527778</v>
+        <v>46157.62644675926</v>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
@@ -3584,31 +3586,33 @@
           <t>03 a 05 dias</t>
         </is>
       </c>
-      <c r="H17" s="5" t="n">
-        <v>2119553175</v>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>OMWVPM</t>
+        </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>MAX SENA DO O</t>
+          <t>VAN LEIJDEN/GUILHERME</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="M17" s="6" t="n">
-        <v>46134.43611111111</v>
+        <v>46157.07361111111</v>
       </c>
       <c r="N17" s="5" t="inlineStr">
         <is>
@@ -3627,17 +3631,17 @@
       </c>
       <c r="Q17" s="5" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="R17" s="5" t="inlineStr">
         <is>
-          <t>Pagamento direto</t>
+          <t>Faturado</t>
         </is>
       </c>
       <c r="S17" s="5" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Aéreo</t>
         </is>
       </c>
       <c r="T17" s="5" t="inlineStr">
@@ -3647,12 +3651,12 @@
       </c>
       <c r="U17" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Independente</t>
         </is>
       </c>
       <c r="V17" s="5" t="inlineStr">
         <is>
-          <t>Jmn Nantes Servicos Financeiros Ltda</t>
+          <t>Tap Air Portugal</t>
         </is>
       </c>
       <c r="W17" s="5" t="inlineStr">
@@ -3662,12 +3666,12 @@
       </c>
       <c r="X17" s="5" t="inlineStr">
         <is>
-          <t>Trend</t>
+          <t>Gol Linhas Aereas</t>
         </is>
       </c>
       <c r="Y17" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>OMWVPM</t>
         </is>
       </c>
       <c r="Z17" s="5" t="inlineStr">
@@ -3681,10 +3685,10 @@
         </is>
       </c>
       <c r="AB17" s="5" t="n">
-        <v>1351</v>
+        <v>610.5</v>
       </c>
       <c r="AC17" s="5" t="n">
-        <v>0</v>
+        <v>52.72</v>
       </c>
       <c r="AD17" s="5" t="n">
         <v>0</v>
@@ -3699,16 +3703,16 @@
         <v>0</v>
       </c>
       <c r="AH17" s="5" t="n">
-        <v>0</v>
+        <v>65.93000000000001</v>
       </c>
       <c r="AI17" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>obs</t>
         </is>
       </c>
       <c r="AJ17" s="5" t="inlineStr">
         <is>
-          <t>Necessário cadastrar um contrato para o cliente ""</t>
+          <t>Centro de custo não preenchido! (ACC01)</t>
         </is>
       </c>
       <c r="AK17" s="5" t="inlineStr">
@@ -3718,12 +3722,12 @@
       </c>
       <c r="AL17" s="5" t="inlineStr">
         <is>
-          <t>Contrato de fornecedor</t>
+          <t>Centro de custo</t>
         </is>
       </c>
       <c r="AM17" s="5" t="inlineStr">
         <is>
-          <t>Análise Cadastro</t>
+          <t>Falta de informação Gerencial</t>
         </is>
       </c>
       <c r="AN17" s="5" t="inlineStr">
@@ -3749,10 +3753,10 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
-        <v>24493444</v>
+        <v>24599722</v>
       </c>
       <c r="B18" s="5" t="n">
-        <v>25304820</v>
+        <v>25425769</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
@@ -3760,10 +3764,10 @@
         </is>
       </c>
       <c r="D18" s="6" t="n">
-        <v>46136.41921296297</v>
+        <v>46157.60678240741</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>46136.42413194444</v>
+        <v>46157.60888888889</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
@@ -3775,31 +3779,33 @@
           <t>03 a 05 dias</t>
         </is>
       </c>
-      <c r="H18" s="5" t="n">
-        <v>2119553171</v>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>YKRRWP</t>
+        </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>MAX SENA DO O</t>
+          <t>VAN LEIJDEN/GUILHERME</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="M18" s="6" t="n">
-        <v>46134.41875</v>
+        <v>46157.06944444445</v>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
@@ -3818,17 +3824,17 @@
       </c>
       <c r="Q18" s="5" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="R18" s="5" t="inlineStr">
         <is>
-          <t>Pagamento direto</t>
+          <t>Faturado</t>
         </is>
       </c>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Aéreo</t>
         </is>
       </c>
       <c r="T18" s="5" t="inlineStr">
@@ -3838,12 +3844,12 @@
       </c>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Independente</t>
         </is>
       </c>
       <c r="V18" s="5" t="inlineStr">
         <is>
-          <t>Jmn Nantes Servicos Financeiros Ltda</t>
+          <t>Tap Air Portugal</t>
         </is>
       </c>
       <c r="W18" s="5" t="inlineStr">
@@ -3853,13 +3859,11 @@
       </c>
       <c r="X18" s="5" t="inlineStr">
         <is>
-          <t>Trend</t>
-        </is>
-      </c>
-      <c r="Y18" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Azul Linhas Aereas</t>
+        </is>
+      </c>
+      <c r="Y18" s="5" t="n">
+        <v>704562481</v>
       </c>
       <c r="Z18" s="5" t="inlineStr">
         <is>
@@ -3872,10 +3876,10 @@
         </is>
       </c>
       <c r="AB18" s="5" t="n">
-        <v>355</v>
+        <v>144</v>
       </c>
       <c r="AC18" s="5" t="n">
-        <v>17.75</v>
+        <v>120.44</v>
       </c>
       <c r="AD18" s="5" t="n">
         <v>0</v>
@@ -3890,16 +3894,16 @@
         <v>0</v>
       </c>
       <c r="AH18" s="5" t="n">
-        <v>0</v>
+        <v>17.28</v>
       </c>
       <c r="AI18" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>obs</t>
         </is>
       </c>
       <c r="AJ18" s="5" t="inlineStr">
         <is>
-          <t>Necessário cadastrar um contrato para o cliente ""</t>
+          <t>Centro de custo não preenchido! (ACC01)</t>
         </is>
       </c>
       <c r="AK18" s="5" t="inlineStr">
@@ -3909,12 +3913,12 @@
       </c>
       <c r="AL18" s="5" t="inlineStr">
         <is>
-          <t>Contrato de fornecedor</t>
+          <t>Centro de custo</t>
         </is>
       </c>
       <c r="AM18" s="5" t="inlineStr">
         <is>
-          <t>Análise Cadastro</t>
+          <t>Falta de informação Gerencial</t>
         </is>
       </c>
       <c r="AN18" s="5" t="inlineStr">
@@ -3940,57 +3944,59 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>24418477</v>
+        <v>24599727</v>
       </c>
       <c r="B19" s="5" t="n">
-        <v>25220450</v>
+        <v>25425774</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D19" s="6" t="n">
-        <v>46120.55074074074</v>
+        <v>46157.60819444444</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>46120.55611111111</v>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>16 a 23 dias</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>16 a 23 dias</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="n">
-        <v>2119510634</v>
+        <v>46157.60957175926</v>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>03 a 05 dias</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>03 a 05 dias</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>UN2CUW</t>
+        </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>JOAO RENATO CUNHA DA SILVA</t>
+          <t>VAN LEIJDEN/GUILHERME</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Kontrip</t>
         </is>
       </c>
       <c r="M19" s="6" t="n">
-        <v>46119.55069444444</v>
+        <v>46157.07569444444</v>
       </c>
       <c r="N19" s="5" t="inlineStr">
         <is>
@@ -4009,17 +4015,17 @@
       </c>
       <c r="Q19" s="5" t="inlineStr">
         <is>
-          <t>Múltiplos</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="R19" s="5" t="inlineStr">
         <is>
-          <t>Múltiplos</t>
+          <t>Faturado</t>
         </is>
       </c>
       <c r="S19" s="5" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Aéreo</t>
         </is>
       </c>
       <c r="T19" s="5" t="inlineStr">
@@ -4029,12 +4035,12 @@
       </c>
       <c r="U19" s="5" t="inlineStr">
         <is>
-          <t>Grupo Kontrip</t>
+          <t>Independente</t>
         </is>
       </c>
       <c r="V19" s="5" t="inlineStr">
         <is>
-          <t>Cogny Solutions Ltda</t>
+          <t>Tap Air Portugal</t>
         </is>
       </c>
       <c r="W19" s="5" t="inlineStr">
@@ -4044,13 +4050,11 @@
       </c>
       <c r="X19" s="5" t="inlineStr">
         <is>
-          <t>Trend</t>
-        </is>
-      </c>
-      <c r="Y19" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Azul Linhas Aereas</t>
+        </is>
+      </c>
+      <c r="Y19" s="5" t="n">
+        <v>802886655</v>
       </c>
       <c r="Z19" s="5" t="inlineStr">
         <is>
@@ -4063,10 +4067,10 @@
         </is>
       </c>
       <c r="AB19" s="5" t="n">
-        <v>951.88</v>
+        <v>108</v>
       </c>
       <c r="AC19" s="5" t="n">
-        <v>43.55</v>
+        <v>106.1</v>
       </c>
       <c r="AD19" s="5" t="n">
         <v>0</v>
@@ -4081,16 +4085,16 @@
         <v>0</v>
       </c>
       <c r="AH19" s="5" t="n">
-        <v>0</v>
+        <v>12.96</v>
       </c>
       <c r="AI19" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>obs</t>
         </is>
       </c>
       <c r="AJ19" s="5" t="inlineStr">
         <is>
-          <t>A soma das tarifas dos registros múltiplos ultrapassa a tarifa da accounting</t>
+          <t>Centro de custo não preenchido! (ACC01)</t>
         </is>
       </c>
       <c r="AK19" s="5" t="inlineStr">
@@ -4100,17 +4104,17 @@
       </c>
       <c r="AL19" s="5" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>Centro de custo</t>
         </is>
       </c>
       <c r="AM19" s="5" t="inlineStr">
         <is>
-          <t>Análise Benner</t>
+          <t>Falta de informação Gerencial</t>
         </is>
       </c>
       <c r="AN19" s="5" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Dados do Fornecedor</t>
         </is>
       </c>
       <c r="AO19" s="5" t="inlineStr">
@@ -4131,10 +4135,10 @@
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
-        <v>24411669</v>
+        <v>24596497</v>
       </c>
       <c r="B20" s="5" t="n">
-        <v>25212946</v>
+        <v>25422131</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
@@ -4142,53 +4146,51 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>46119.44847222222</v>
+        <v>46156.82958333333</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>46121.62430555555</v>
-      </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>16 a 23 dias</t>
-        </is>
-      </c>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>16 a 23 dias</t>
+        <v>46157.08439814814</v>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>03 a 05 dias</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>MV1MCEMYDABR</t>
+          <t>FAPDBO</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>WOOBA</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>MAX SENA DO O</t>
+          <t>CAMANO DE MESQUITA BARROS/LUCAS MR</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Toou</t>
         </is>
       </c>
       <c r="L20" s="5" t="inlineStr">
         <is>
-          <t>Emilly Tavares Santos</t>
+          <t>Toou</t>
         </is>
       </c>
       <c r="M20" s="6" t="n">
-        <v>46118.44791666666</v>
-      </c>
-      <c r="N20" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>46156.82847222222</v>
+      </c>
+      <c r="N20" s="5" t="n">
+        <v>2340</v>
       </c>
       <c r="O20" s="5" t="inlineStr">
         <is>
@@ -4202,17 +4204,17 @@
       </c>
       <c r="Q20" s="5" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="R20" s="5" t="inlineStr">
         <is>
-          <t>Pagamento direto</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="S20" s="5" t="inlineStr">
         <is>
-          <t>Carro</t>
+          <t>Aéreo</t>
         </is>
       </c>
       <c r="T20" s="5" t="inlineStr">
@@ -4222,12 +4224,12 @@
       </c>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Independente</t>
         </is>
       </c>
       <c r="V20" s="5" t="inlineStr">
         <is>
-          <t>Jmn Nantes Servicos Financeiros Ltda</t>
+          <t>Projetech Locacao</t>
         </is>
       </c>
       <c r="W20" s="5" t="inlineStr">
@@ -4237,13 +4239,11 @@
       </c>
       <c r="X20" s="5" t="inlineStr">
         <is>
-          <t>Movida - Br - Sp - Sao Paulo - Itaim Bibi</t>
-        </is>
-      </c>
-      <c r="Y20" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Latam Airlines Brasil</t>
+        </is>
+      </c>
+      <c r="Y20" s="5" t="n">
+        <v>2286806156</v>
       </c>
       <c r="Z20" s="5" t="inlineStr">
         <is>
@@ -4256,10 +4256,10 @@
         </is>
       </c>
       <c r="AB20" s="5" t="n">
-        <v>660.03</v>
+        <v>814.5599999999999</v>
       </c>
       <c r="AC20" s="5" t="n">
-        <v>0</v>
+        <v>72.03</v>
       </c>
       <c r="AD20" s="5" t="n">
         <v>0</v>
@@ -4274,11 +4274,11 @@
         <v>0</v>
       </c>
       <c r="AH20" s="5" t="n">
-        <v>0</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="AI20" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Reserva importada do Sistema WOOBA. Id: 5966</t>
         </is>
       </c>
       <c r="AJ20" s="5" t="inlineStr">
@@ -4317,199 +4317,6 @@
         </is>
       </c>
       <c r="AQ20" s="5" t="inlineStr">
-        <is>
-          <t>Operações - KONTRIP</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="n">
-        <v>24495479</v>
-      </c>
-      <c r="B21" s="5" t="n">
-        <v>25307271</v>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>ACC01</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="n">
-        <v>46136.7365625</v>
-      </c>
-      <c r="E21" s="6" t="n">
-        <v>46136.75099537037</v>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>03 a 05 dias</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>03 a 05 dias</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>MV1JTTDQJ1BR</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>MANUAL</t>
-        </is>
-      </c>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>RUBENS OSTERNACK FILHO</t>
-        </is>
-      </c>
-      <c r="K21" s="5" t="inlineStr">
-        <is>
-          <t>Emilly Tavares Santos</t>
-        </is>
-      </c>
-      <c r="L21" s="5" t="inlineStr">
-        <is>
-          <t>Emilly Tavares Santos</t>
-        </is>
-      </c>
-      <c r="M21" s="6" t="n">
-        <v>46128.73611111111</v>
-      </c>
-      <c r="N21" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O21" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P21" s="5" t="inlineStr">
-        <is>
-          <t>OFF LINE</t>
-        </is>
-      </c>
-      <c r="Q21" s="5" t="inlineStr">
-        <is>
-          <t>Outros</t>
-        </is>
-      </c>
-      <c r="R21" s="5" t="inlineStr">
-        <is>
-          <t>Pagamento direto</t>
-        </is>
-      </c>
-      <c r="S21" s="5" t="inlineStr">
-        <is>
-          <t>Carro</t>
-        </is>
-      </c>
-      <c r="T21" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="U21" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V21" s="5" t="inlineStr">
-        <is>
-          <t>Jmn Nantes Servicos Financeiros Ltda</t>
-        </is>
-      </c>
-      <c r="W21" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X21" s="5" t="inlineStr">
-        <is>
-          <t>Movida - Br - Sp - Sao Paulo - Itaim Bibi - Matriz</t>
-        </is>
-      </c>
-      <c r="Y21" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z21" s="5" t="inlineStr">
-        <is>
-          <t>KONTRIP</t>
-        </is>
-      </c>
-      <c r="AA21" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB21" s="5" t="n">
-        <v>909.36</v>
-      </c>
-      <c r="AC21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI21" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AJ21" s="5" t="inlineStr">
-        <is>
-          <t>Necessário cadastrar um contrato para o cliente ""</t>
-        </is>
-      </c>
-      <c r="AK21" s="5" t="inlineStr">
-        <is>
-          <t>KONTRIP</t>
-        </is>
-      </c>
-      <c r="AL21" s="5" t="inlineStr">
-        <is>
-          <t>Contrato de fornecedor</t>
-        </is>
-      </c>
-      <c r="AM21" s="5" t="inlineStr">
-        <is>
-          <t>Análise Cadastro</t>
-        </is>
-      </c>
-      <c r="AN21" s="5" t="inlineStr">
-        <is>
-          <t>Dados do Fornecedor</t>
-        </is>
-      </c>
-      <c r="AO21" s="5" t="inlineStr">
-        <is>
-          <t>Qualidade dos dados</t>
-        </is>
-      </c>
-      <c r="AP21" s="5" t="inlineStr">
-        <is>
-          <t>KONTRIP VIAGENS</t>
-        </is>
-      </c>
-      <c r="AQ21" s="5" t="inlineStr">
         <is>
           <t>Operações - KONTRIP</t>
         </is>

</xml_diff>